<commit_message>
Add the generated questions for OS CA DB in excel file by automating the process
</commit_message>
<xml_diff>
--- a/dataset/outputs/P000233DS_Question_Dataset.xlsx
+++ b/dataset/outputs/P000233DS_Question_Dataset.xlsx
@@ -2,15 +2,14 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Question Dataset" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -28,7 +27,7 @@
     <font>
       <name val="Arial"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
       <sz val="10"/>
     </font>
     <font>
@@ -36,7 +35,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -45,7 +44,22 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F4E79"/>
+        <fgColor rgb="FF1F4E79"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEBF3FB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EBF3FB"/>
       </patternFill>
     </fill>
     <fill>
@@ -53,17 +67,71 @@
         <fgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00EBF3FB"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="6">
+  <borders count="7">
     <border>
       <left/>
       <right/>
       <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFCCCCCC"/>
+      </top>
       <bottom/>
       <diagonal/>
     </border>
@@ -81,55 +149,11 @@
         <color rgb="00CCCCCC"/>
       </bottom>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="00CCCCCC"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="00CCCCCC"/>
-      </right>
-      <top style="thin">
-        <color rgb="00CCCCCC"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color rgb="00CCCCCC"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00CCCCCC"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color rgb="00CCCCCC"/>
-      </right>
-      <top style="thin">
-        <color rgb="00CCCCCC"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00CCCCCC"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -140,11 +164,20 @@
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -507,8 +540,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T17"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:T62"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5" outlineLevelCol="0"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
@@ -518,167 +551,163 @@
     <col width="16" customWidth="1" min="6" max="6"/>
     <col width="8" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="50" customWidth="1" min="9" max="9"/>
-    <col width="50" customWidth="1" min="10" max="10"/>
+    <col width="50" customWidth="1" min="9" max="10"/>
     <col width="25" customWidth="1" min="11" max="11"/>
-    <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="12" customWidth="1" min="13" max="13"/>
-    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="12" max="14"/>
     <col width="10" customWidth="1" min="15" max="15"/>
-    <col width="14" customWidth="1" min="16" max="16"/>
-    <col width="14" customWidth="1" min="17" max="17"/>
+    <col width="14" customWidth="1" min="16" max="17"/>
     <col width="35" customWidth="1" min="18" max="18"/>
     <col width="18" customWidth="1" min="19" max="19"/>
     <col width="12" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>INPUT PARAMETERS</t>
         </is>
       </c>
-      <c r="B1" s="4" t="n"/>
-      <c r="C1" s="4" t="n"/>
-      <c r="D1" s="5" t="n"/>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="B1" s="5" t="n"/>
+      <c r="C1" s="5" t="n"/>
+      <c r="D1" s="6" t="n"/>
+      <c r="E1" s="4" t="inlineStr">
         <is>
           <t>RAG CONFIGURATION</t>
         </is>
       </c>
-      <c r="F1" s="4" t="n"/>
-      <c r="G1" s="4" t="n"/>
-      <c r="H1" s="5" t="n"/>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="F1" s="5" t="n"/>
+      <c r="G1" s="5" t="n"/>
+      <c r="H1" s="6" t="n"/>
+      <c r="I1" s="4" t="inlineStr">
         <is>
           <t>GENERATED OUTPUT</t>
         </is>
       </c>
-      <c r="J1" s="4" t="n"/>
-      <c r="K1" s="5" t="n"/>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="J1" s="5" t="n"/>
+      <c r="K1" s="6" t="n"/>
+      <c r="L1" s="4" t="inlineStr">
         <is>
           <t>LLM JUDGE SCORES</t>
         </is>
       </c>
-      <c r="M1" s="4" t="n"/>
-      <c r="N1" s="4" t="n"/>
-      <c r="O1" s="5" t="n"/>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="M1" s="5" t="n"/>
+      <c r="N1" s="5" t="n"/>
+      <c r="O1" s="6" t="n"/>
+      <c r="P1" s="4" t="inlineStr">
         <is>
           <t>HUMAN REVIEW</t>
         </is>
       </c>
-      <c r="Q1" s="5" t="n"/>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="Q1" s="6" t="n"/>
+      <c r="R1" s="4" t="inlineStr">
         <is>
           <t>REMARKS</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" s="4" t="inlineStr">
         <is>
           <t>META</t>
         </is>
       </c>
-      <c r="T1" s="5" t="n"/>
+      <c r="T1" s="6" t="n"/>
     </row>
     <row r="2" ht="35" customHeight="1">
-      <c r="A2" s="1" t="inlineStr">
+      <c r="A2" s="4" t="inlineStr">
         <is>
           <t>Q_ID</t>
         </is>
       </c>
-      <c r="B2" s="1" t="inlineStr">
+      <c r="B2" s="4" t="inlineStr">
         <is>
           <t>Domain</t>
         </is>
       </c>
-      <c r="C2" s="1" t="inlineStr">
+      <c r="C2" s="4" t="inlineStr">
         <is>
           <t>Difficulty</t>
         </is>
       </c>
-      <c r="D2" s="1" t="inlineStr">
+      <c r="D2" s="4" t="inlineStr">
         <is>
           <t>Question Type</t>
         </is>
       </c>
-      <c r="E2" s="1" t="inlineStr">
+      <c r="E2" s="4" t="inlineStr">
         <is>
           <t>Learning Objective</t>
         </is>
       </c>
-      <c r="F2" s="1" t="inlineStr">
+      <c r="F2" s="4" t="inlineStr">
         <is>
           <t>Routing Method</t>
         </is>
       </c>
-      <c r="G2" s="1" t="inlineStr">
+      <c r="G2" s="4" t="inlineStr">
         <is>
           <t>Top K</t>
         </is>
       </c>
-      <c r="H2" s="1" t="inlineStr">
+      <c r="H2" s="4" t="inlineStr">
         <is>
           <t>Seed Ratio</t>
         </is>
       </c>
-      <c r="I2" s="1" t="inlineStr">
+      <c r="I2" s="4" t="inlineStr">
         <is>
           <t>Generated Question</t>
         </is>
       </c>
-      <c r="J2" s="1" t="inlineStr">
+      <c r="J2" s="4" t="inlineStr">
         <is>
           <t>Sample Answer</t>
         </is>
       </c>
-      <c r="K2" s="1" t="inlineStr">
+      <c r="K2" s="4" t="inlineStr">
         <is>
           <t>Sources Used</t>
         </is>
       </c>
-      <c r="L2" s="1" t="inlineStr">
+      <c r="L2" s="4" t="inlineStr">
         <is>
           <t>Q Score (/5)</t>
         </is>
       </c>
-      <c r="M2" s="1" t="inlineStr">
+      <c r="M2" s="4" t="inlineStr">
         <is>
           <t>A Score (/5)</t>
         </is>
       </c>
-      <c r="N2" s="1" t="inlineStr">
+      <c r="N2" s="4" t="inlineStr">
         <is>
           <t>R Score (/5)</t>
         </is>
       </c>
-      <c r="O2" s="1" t="inlineStr">
+      <c r="O2" s="4" t="inlineStr">
         <is>
           <t>Attempts</t>
         </is>
       </c>
-      <c r="P2" s="1" t="inlineStr">
+      <c r="P2" s="4" t="inlineStr">
         <is>
           <t>Human Rating</t>
         </is>
       </c>
-      <c r="Q2" s="1" t="inlineStr">
+      <c r="Q2" s="4" t="inlineStr">
         <is>
           <t>Reviewed By</t>
         </is>
       </c>
-      <c r="R2" s="1" t="inlineStr">
+      <c r="R2" s="4" t="inlineStr">
         <is>
           <t>Remarks</t>
         </is>
       </c>
-      <c r="S2" s="1" t="inlineStr">
+      <c r="S2" s="4" t="inlineStr">
         <is>
           <t>Generated At</t>
         </is>
       </c>
-      <c r="T2" s="1" t="inlineStr">
+      <c r="T2" s="4" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
@@ -752,9 +781,9 @@
       <c r="O3" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="P3" s="2" t="inlineStr"/>
-      <c r="Q3" s="2" t="inlineStr"/>
-      <c r="R3" s="2" t="inlineStr"/>
+      <c r="P3" s="2" t="n"/>
+      <c r="Q3" s="2" t="n"/>
+      <c r="R3" s="2" t="n"/>
       <c r="S3" s="2" t="inlineStr">
         <is>
           <t>2026-05-15 04:48</t>
@@ -834,9 +863,9 @@
       <c r="O4" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="P4" s="3" t="inlineStr"/>
-      <c r="Q4" s="3" t="inlineStr"/>
-      <c r="R4" s="3" t="inlineStr"/>
+      <c r="P4" s="3" t="n"/>
+      <c r="Q4" s="3" t="n"/>
+      <c r="R4" s="3" t="n"/>
       <c r="S4" s="3" t="inlineStr">
         <is>
           <t>2026-05-15 04:49</t>
@@ -914,9 +943,9 @@
       <c r="O5" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="P5" s="2" t="inlineStr"/>
-      <c r="Q5" s="2" t="inlineStr"/>
-      <c r="R5" s="2" t="inlineStr"/>
+      <c r="P5" s="2" t="n"/>
+      <c r="Q5" s="2" t="n"/>
+      <c r="R5" s="2" t="n"/>
       <c r="S5" s="2" t="inlineStr">
         <is>
           <t>2026-05-15 04:49</t>
@@ -994,9 +1023,9 @@
       <c r="O6" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="P6" s="3" t="inlineStr"/>
-      <c r="Q6" s="3" t="inlineStr"/>
-      <c r="R6" s="3" t="inlineStr"/>
+      <c r="P6" s="3" t="n"/>
+      <c r="Q6" s="3" t="n"/>
+      <c r="R6" s="3" t="n"/>
       <c r="S6" s="3" t="inlineStr">
         <is>
           <t>2026-05-15 04:50</t>
@@ -1076,9 +1105,9 @@
       <c r="O7" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="P7" s="2" t="inlineStr"/>
-      <c r="Q7" s="2" t="inlineStr"/>
-      <c r="R7" s="2" t="inlineStr"/>
+      <c r="P7" s="2" t="n"/>
+      <c r="Q7" s="2" t="n"/>
+      <c r="R7" s="2" t="n"/>
       <c r="S7" s="2" t="inlineStr">
         <is>
           <t>2026-05-15 04:51</t>
@@ -1158,9 +1187,9 @@
       <c r="O8" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="P8" s="3" t="inlineStr"/>
-      <c r="Q8" s="3" t="inlineStr"/>
-      <c r="R8" s="3" t="inlineStr"/>
+      <c r="P8" s="3" t="n"/>
+      <c r="Q8" s="3" t="n"/>
+      <c r="R8" s="3" t="n"/>
       <c r="S8" s="3" t="inlineStr">
         <is>
           <t>2026-05-15 04:51</t>
@@ -1240,9 +1269,9 @@
       <c r="O9" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="P9" s="2" t="inlineStr"/>
-      <c r="Q9" s="2" t="inlineStr"/>
-      <c r="R9" s="2" t="inlineStr"/>
+      <c r="P9" s="2" t="n"/>
+      <c r="Q9" s="2" t="n"/>
+      <c r="R9" s="2" t="n"/>
       <c r="S9" s="2" t="inlineStr">
         <is>
           <t>2026-05-15 04:52</t>
@@ -1322,9 +1351,9 @@
       <c r="O10" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="P10" s="3" t="inlineStr"/>
-      <c r="Q10" s="3" t="inlineStr"/>
-      <c r="R10" s="3" t="inlineStr"/>
+      <c r="P10" s="3" t="n"/>
+      <c r="Q10" s="3" t="n"/>
+      <c r="R10" s="3" t="n"/>
       <c r="S10" s="3" t="inlineStr">
         <is>
           <t>2026-05-15 04:52</t>
@@ -1404,9 +1433,9 @@
       <c r="O11" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="P11" s="2" t="inlineStr"/>
-      <c r="Q11" s="2" t="inlineStr"/>
-      <c r="R11" s="2" t="inlineStr"/>
+      <c r="P11" s="2" t="n"/>
+      <c r="Q11" s="2" t="n"/>
+      <c r="R11" s="2" t="n"/>
       <c r="S11" s="2" t="inlineStr">
         <is>
           <t>2026-05-15 04:53</t>
@@ -1486,9 +1515,9 @@
       <c r="O12" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="P12" s="3" t="inlineStr"/>
-      <c r="Q12" s="3" t="inlineStr"/>
-      <c r="R12" s="3" t="inlineStr"/>
+      <c r="P12" s="3" t="n"/>
+      <c r="Q12" s="3" t="n"/>
+      <c r="R12" s="3" t="n"/>
       <c r="S12" s="3" t="inlineStr">
         <is>
           <t>2026-05-15 04:54</t>
@@ -1568,9 +1597,9 @@
       <c r="O13" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="P13" s="3" t="inlineStr"/>
-      <c r="Q13" s="3" t="inlineStr"/>
-      <c r="R13" s="3" t="inlineStr"/>
+      <c r="P13" s="3" t="n"/>
+      <c r="Q13" s="3" t="n"/>
+      <c r="R13" s="3" t="n"/>
       <c r="S13" s="3" t="inlineStr">
         <is>
           <t>2026-05-15 04:56</t>
@@ -1650,9 +1679,9 @@
       <c r="O14" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="P14" s="2" t="inlineStr"/>
-      <c r="Q14" s="2" t="inlineStr"/>
-      <c r="R14" s="2" t="inlineStr"/>
+      <c r="P14" s="2" t="n"/>
+      <c r="Q14" s="2" t="n"/>
+      <c r="R14" s="2" t="n"/>
       <c r="S14" s="2" t="inlineStr">
         <is>
           <t>2026-05-15 04:56</t>
@@ -1736,9 +1765,9 @@
       <c r="O15" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="P15" s="2" t="inlineStr"/>
-      <c r="Q15" s="2" t="inlineStr"/>
-      <c r="R15" s="2" t="inlineStr"/>
+      <c r="P15" s="2" t="n"/>
+      <c r="Q15" s="2" t="n"/>
+      <c r="R15" s="2" t="n"/>
       <c r="S15" s="2" t="inlineStr">
         <is>
           <t>2026-05-16 12:55</t>
@@ -1822,9 +1851,9 @@
       <c r="O16" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="P16" s="3" t="inlineStr"/>
-      <c r="Q16" s="3" t="inlineStr"/>
-      <c r="R16" s="3" t="inlineStr"/>
+      <c r="P16" s="3" t="n"/>
+      <c r="Q16" s="3" t="n"/>
+      <c r="R16" s="3" t="n"/>
       <c r="S16" s="3" t="inlineStr">
         <is>
           <t>2026-05-16 12:55</t>
@@ -1904,15 +1933,3706 @@
       <c r="O17" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="P17" s="2" t="inlineStr"/>
-      <c r="Q17" s="2" t="inlineStr"/>
-      <c r="R17" s="2" t="inlineStr"/>
+      <c r="P17" s="2" t="n"/>
+      <c r="Q17" s="2" t="n"/>
+      <c r="R17" s="2" t="n"/>
       <c r="S17" s="2" t="inlineStr">
         <is>
           <t>2026-05-16 12:56</t>
         </is>
       </c>
       <c r="T17" s="2" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="80" customHeight="1">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>E-DA-016</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>database</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>recall</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>Database normalisation</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>explicit</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H18" s="3" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="I18" s="3" t="inlineStr">
+        <is>
+          <t>What does the term "further restructurings of conceptual schemas" refer to in the context of database design, and provide an example scenario where such restructurings might be necessary?</t>
+        </is>
+      </c>
+      <c r="J18" s="3" t="inlineStr">
+        <is>
+          <t>Further restructurings of conceptual schemas refer to adjustments made to the initial design of a database schema when certain relations cannot be effectively decomposed into Boyce-Codd normal form. For instance, if a schema including students, their degree programmes, and supervising professors results in a relation that fails to meet the criteria for normalization, restructuring may be necessary to better organize the data and ensure it meets the required functional dependencies.</t>
+        </is>
+      </c>
+      <c r="K18" s="3" t="inlineStr">
+        <is>
+          <t>source_8.pdf, source_31.pdf, source_7.pdf, source_36.pdf, source_49.pdf, source_13.pdf, source_14.pdf</t>
+        </is>
+      </c>
+      <c r="L18" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="M18" s="3" t="n">
+        <v>4.75</v>
+      </c>
+      <c r="N18" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="O18" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="P18" s="3" t="n"/>
+      <c r="Q18" s="3" t="n"/>
+      <c r="R18" s="3" t="n"/>
+      <c r="S18" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-16 13:09</t>
+        </is>
+      </c>
+      <c r="T18" s="3" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="80" customHeight="1">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>E-DA-017</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>database</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>recall</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>SQL joins — inner and outer</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>explicit</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>Which SQL statement would produce a result set that includes all rows from both tables, even if there is no match between them?</t>
+        </is>
+      </c>
+      <c r="J19" s="2" t="inlineStr">
+        <is>
+          <t>A SQL statement that would produce a result set including all rows from both tables, even if there is no match between them, utilizes a FULL OUTER JOIN. This join type combines all records from both tables, adding rows with NULL values for columns from the non-matching table where no corresponding record exists in either table.</t>
+        </is>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>source_8.pdf, source_31.pdf, source_7.pdf, source_36.pdf, source_49.pdf, source_13.pdf, source_14.pdf</t>
+        </is>
+      </c>
+      <c r="L19" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="M19" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="N19" s="2" t="n">
+        <v>1.67</v>
+      </c>
+      <c r="O19" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="P19" s="2" t="n"/>
+      <c r="Q19" s="2" t="n"/>
+      <c r="R19" s="2" t="n"/>
+      <c r="S19" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-16 13:09</t>
+        </is>
+      </c>
+      <c r="T19" s="2" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="80" customHeight="1">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>E-DA-018</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>database</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>recall</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>ACID properties in database transactions</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>explicit</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H20" s="3" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="I20" s="3" t="inlineStr">
+        <is>
+          <t>What does the term "acid properties" refer to in the context of database transactions?</t>
+        </is>
+      </c>
+      <c r="J20" s="3" t="inlineStr">
+        <is>
+          <t>The term "acid properties" refers to the four essential characteristics that transactions in a database management system must exhibit: atomicity, consistency, isolation, and durability. These properties ensure that transactions are processed reliably and maintain the integrity of the database, making them crucial for the proper functioning of database systems.</t>
+        </is>
+      </c>
+      <c r="K20" s="3" t="inlineStr">
+        <is>
+          <t>source_8.pdf, source_31.pdf, source_7.pdf, source_17.pdf, source_36.pdf, source_49.pdf, source_13.pdf, source_18.pdf</t>
+        </is>
+      </c>
+      <c r="L20" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="M20" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="N20" s="3" t="n">
+        <v>1.67</v>
+      </c>
+      <c r="O20" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="P20" s="3" t="n"/>
+      <c r="Q20" s="3" t="n"/>
+      <c r="R20" s="3" t="n"/>
+      <c r="S20" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-16 13:10</t>
+        </is>
+      </c>
+      <c r="T20" s="3" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="80" customHeight="1">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>E-DA-019</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>database</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>recall</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>Transaction management and concurrency</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>explicit</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>What does the x-open dtp standard allow for in terms of resource managers (rms)?</t>
+        </is>
+      </c>
+      <c r="J21" s="2" t="inlineStr">
+        <is>
+          <t>The X/Open DTP standard allows for totally passive resource managers (RMs), where all protocol control is centralized within the transaction manager (TM), which activates RM functions through a library of remotely callable primitives.</t>
+        </is>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>source_8.pdf, source_31.pdf, source_7.pdf, source_17.pdf, source_36.pdf, source_49.pdf, source_13.pdf, source_14.pdf, source_18.pdf</t>
+        </is>
+      </c>
+      <c r="L21" s="2" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="M21" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="N21" s="2" t="n">
+        <v>1.67</v>
+      </c>
+      <c r="O21" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="P21" s="2" t="n"/>
+      <c r="Q21" s="2" t="n"/>
+      <c r="R21" s="2" t="n"/>
+      <c r="S21" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-16 13:12</t>
+        </is>
+      </c>
+      <c r="T21" s="2" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="80" customHeight="1">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>E-DA-020</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>database</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>recall</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>Indexing and query optimisation</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>explicit</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H22" s="3" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="I22" s="3" t="inlineStr">
+        <is>
+          <t>What does the final part (page trailer) of a data page typically contain, and what is its purpose in relation to indexe?</t>
+        </is>
+      </c>
+      <c r="J22" s="3" t="inlineStr">
+        <is>
+          <t>The final part (page trailer) of a data page typically contains control information such as identifiers for objects like tables or indexes, pointers to adjacent pages, and metadata about the number of tuples stored on the page and available memory. This information supports efficient management and access to index structures by enabling quick location and navigation through the database pages.</t>
+        </is>
+      </c>
+      <c r="K22" s="3" t="inlineStr">
+        <is>
+          <t>source_8.pdf, source_31.pdf, source_7.pdf, source_50.pdf, source_36.pdf, source_49.pdf, source_13.pdf, source_14.pdf, source_18.pdf</t>
+        </is>
+      </c>
+      <c r="L22" s="3" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="M22" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="N22" s="3" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="O22" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="P22" s="3" t="n"/>
+      <c r="Q22" s="3" t="n"/>
+      <c r="R22" s="3" t="n"/>
+      <c r="S22" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-16 13:12</t>
+        </is>
+      </c>
+      <c r="T22" s="3" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="80" customHeight="1">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>E-DA-021</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>database</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>recall</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>Two phase locking and deadlock prevention</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>explicit</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>Which of the following statements best describes the concept of serializability in the context of transaction scheduling?
+In the given schedule, how does the two-phase locking mechanism ensure that the final values of A and B are consistent from any consistent initial state?</t>
+        </is>
+      </c>
+      <c r="J23" s="2" t="inlineStr">
+        <is>
+          <t>Serializability ensures that a schedule of concurrent transactions appears as if they executed one after another in some order, maintaining the consistency properties of individual transactions. In the given schedule, two-phase locking prevents transactions from holding locks indefinitely and ensures that once a transaction releases a lock, no further updates can occur, thereby preserving consistency from any consistent initial state.</t>
+        </is>
+      </c>
+      <c r="K23" s="2" t="inlineStr">
+        <is>
+          <t>source_7.pdf, source_49.pdf, source_13.pdf, source_8.pdf</t>
+        </is>
+      </c>
+      <c r="L23" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="M23" s="2" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="N23" s="2" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="O23" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="P23" s="2" t="n"/>
+      <c r="Q23" s="2" t="n"/>
+      <c r="R23" s="2" t="n"/>
+      <c r="S23" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-16 13:13</t>
+        </is>
+      </c>
+      <c r="T23" s="2" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="80" customHeight="1">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>E-DA-022</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>database</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>recall</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>Entity relationship modelling</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>explicit</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H24" s="3" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="I24" s="3" t="inlineStr">
+        <is>
+          <t>What is the purpose of creating a relation schema `person` when using the second method for mapping an entity-relationship design to relational schemas?</t>
+        </is>
+      </c>
+      <c r="J24" s="3" t="inlineStr">
+        <is>
+          <t>Creating a relation schema `person` ensures that there is a single relation to which a foreign-key constraint on another relation (R) can refer, thus avoiding the issue of having multiple entities without a clear referencing relation. This is essential for maintaining referential integrity in the relational model when employing the second method for mapping entity-relationship designs to relational schemas.</t>
+        </is>
+      </c>
+      <c r="K24" s="3" t="inlineStr">
+        <is>
+          <t>source_8.pdf, source_31.pdf, source_7.pdf, source_36.pdf, source_49.pdf, source_13.pdf, source_14.pdf</t>
+        </is>
+      </c>
+      <c r="L24" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="M24" s="3" t="n">
+        <v>4.25</v>
+      </c>
+      <c r="N24" s="3" t="n">
+        <v>1.67</v>
+      </c>
+      <c r="O24" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="P24" s="3" t="n"/>
+      <c r="Q24" s="3" t="n"/>
+      <c r="R24" s="3" t="n"/>
+      <c r="S24" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-16 13:14</t>
+        </is>
+      </c>
+      <c r="T24" s="3" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="80" customHeight="1">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>E-DA-023</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>database</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>recall</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>Relational algebra and calculus</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>explicit</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>What operation in relational algebra is used to select tuples that satisfy a given condition from a relation?</t>
+        </is>
+      </c>
+      <c r="J25" s="2" t="inlineStr">
+        <is>
+          <t>The operation in relational algebra used to select tuples that satisfy a given condition from a relation is known as selection. This operation filters the tuples in a relation based on a specified condition, returning only those tuples that meet the criteria defined in the selection condition.</t>
+        </is>
+      </c>
+      <c r="K25" s="2" t="inlineStr">
+        <is>
+          <t>source_8.pdf, source_31.pdf, source_7.pdf, source_17.pdf, source_36.pdf, source_49.pdf, source_13.pdf, source_14.pdf, source_18.pdf</t>
+        </is>
+      </c>
+      <c r="L25" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="M25" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="N25" s="2" t="n">
+        <v>1.67</v>
+      </c>
+      <c r="O25" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="P25" s="2" t="n"/>
+      <c r="Q25" s="2" t="n"/>
+      <c r="R25" s="2" t="n"/>
+      <c r="S25" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-16 13:14</t>
+        </is>
+      </c>
+      <c r="T25" s="2" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="80" customHeight="1">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>E-DA-024</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>database</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>recall</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>Stored procedures and triggers</t>
+        </is>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>explicit</t>
+        </is>
+      </c>
+      <c r="G26" s="3" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H26" s="3" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="I26" s="3" t="inlineStr">
+        <is>
+          <t>What is a trigger and what are its key characteristics?</t>
+        </is>
+      </c>
+      <c r="J26" s="3" t="inlineStr">
+        <is>
+          <t>A trigger is procedural SQL code automatically invoked by the database management system in response to specific data manipulation events such as insertions, updates, or deletions. Key characteristics include being associated with a particular table, capable of executing before or after the triggering event within the same transaction, and potentially having multiple triggers per table.</t>
+        </is>
+      </c>
+      <c r="K26" s="3" t="inlineStr">
+        <is>
+          <t>source_8.pdf, source_31.pdf, source_7.pdf, source_17.pdf, source_36.pdf, source_49.pdf, source_13.pdf, source_18.pdf</t>
+        </is>
+      </c>
+      <c r="L26" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="M26" s="3" t="n">
+        <v>4.25</v>
+      </c>
+      <c r="N26" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="O26" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="P26" s="3" t="n"/>
+      <c r="Q26" s="3" t="n"/>
+      <c r="R26" s="3" t="n"/>
+      <c r="S26" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-16 13:15</t>
+        </is>
+      </c>
+      <c r="T26" s="3" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="80" customHeight="1">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>E-DA-025</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>database</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>recall</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="inlineStr">
+        <is>
+          <t>Database recovery and logging</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>explicit</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>Which book provides a more detailed and comprehensive treatment of recovery and concurrency control compared to the earlier survey by P. A. Bernstein, N. Goodman, and V. Hadzilacos?</t>
+        </is>
+      </c>
+      <c r="J27" s="2" t="inlineStr">
+        <is>
+          <t>The book "Concurrency Control and Recovery in Database Systems" by P. A. Bernstein, V. Hadzilacos, and N. Goodman offers a more detailed and comprehensive treatment of recovery and concurrency control compared to the earlier survey by P. A. Bernstein, N. Goodman, and V. Hadzilacos, as it was published later and represents more recent advancements in the field.</t>
+        </is>
+      </c>
+      <c r="K27" s="2" t="inlineStr">
+        <is>
+          <t>source_8.pdf, source_31.pdf, source_7.pdf, source_17.pdf, source_36.pdf, source_49.pdf, source_13.pdf, source_14.pdf</t>
+        </is>
+      </c>
+      <c r="L27" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="M27" s="2" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="N27" s="2" t="n">
+        <v>1.67</v>
+      </c>
+      <c r="O27" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="P27" s="2" t="n"/>
+      <c r="Q27" s="2" t="n"/>
+      <c r="R27" s="2" t="n"/>
+      <c r="S27" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-16 13:15</t>
+        </is>
+      </c>
+      <c r="T27" s="2" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="80" customHeight="1">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>E-DA-026</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>database</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>recall</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>NoSQL vs relational databases</t>
+        </is>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>explicit</t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H28" s="3" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="I28" s="3" t="inlineStr">
+        <is>
+          <t>What are the pros and cons of using a single table to implement multiple relationships in a database, specifically for the case where T has relationships with both S and U through R and Q, respectively?</t>
+        </is>
+      </c>
+      <c r="J28" s="3" t="inlineStr">
+        <is>
+          <t>Using a single table to implement multiple relationships can streamline data management by reducing the number of tables needed, thus simplifying schema design and potentially improving query performance. However, this approach can also lead to complex schema designs that may become difficult to manage, especially as the number of relationships grows, and it may introduce null values that complicate data integrity and consistency checks.</t>
+        </is>
+      </c>
+      <c r="K28" s="3" t="inlineStr">
+        <is>
+          <t>source_8.pdf, source_31.pdf, source_7.pdf, source_50.pdf, source_36.pdf, source_49.pdf, source_13.pdf, source_14.pdf, source_18.pdf</t>
+        </is>
+      </c>
+      <c r="L28" s="3" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="M28" s="3" t="n">
+        <v>4.25</v>
+      </c>
+      <c r="N28" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="O28" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="P28" s="3" t="n"/>
+      <c r="Q28" s="3" t="n"/>
+      <c r="R28" s="3" t="n"/>
+      <c r="S28" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-16 13:16</t>
+        </is>
+      </c>
+      <c r="T28" s="3" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="80" customHeight="1">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>E-DA-027</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>database</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>recall</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="inlineStr">
+        <is>
+          <t>B-tree and hash indexing</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>explicit</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>What clause is used in SQL queries to apply conditions at the end of the execution of a query that uses the GROUP BY clause?</t>
+        </is>
+      </c>
+      <c r="J29" s="2" t="inlineStr">
+        <is>
+          <t>The having clause is used in SQL queries to apply conditions at the end of the execution of a query that uses the GROUP BY clause. This clause specifies the criteria that each subset of rows forming part of the result must satisfy after the aggregation operations have been executed.</t>
+        </is>
+      </c>
+      <c r="K29" s="2" t="inlineStr">
+        <is>
+          <t>source_8.pdf, source_31.pdf, source_7.pdf, source_36.pdf, source_49.pdf, source_13.pdf, source_14.pdf</t>
+        </is>
+      </c>
+      <c r="L29" s="2" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="M29" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="N29" s="2" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="O29" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="P29" s="2" t="n"/>
+      <c r="Q29" s="2" t="n"/>
+      <c r="R29" s="2" t="n"/>
+      <c r="S29" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-16 13:17</t>
+        </is>
+      </c>
+      <c r="T29" s="2" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="80" customHeight="1">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>E-DA-028</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>database</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>recall</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>Query execution plans and optimiser</t>
+        </is>
+      </c>
+      <c r="F30" s="3" t="inlineStr">
+        <is>
+          <t>explicit</t>
+        </is>
+      </c>
+      <c r="G30" s="3" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H30" s="3" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="I30" s="3" t="inlineStr">
+        <is>
+          <t>What is the title of the paper by G. Graefe and W. McKenna that discusses the Volcano Optimizer Generator?</t>
+        </is>
+      </c>
+      <c r="J30" s="3" t="inlineStr">
+        <is>
+          <t>The title of the paper by G. Graefe and W. McKenna that discusses the Volcano Optimizer Generator is "The Volcano Optimizer Generator", which was presented at the International Conference on Data Engineering in 1993.</t>
+        </is>
+      </c>
+      <c r="K30" s="3" t="inlineStr">
+        <is>
+          <t>source_7.pdf, source_49.pdf, source_8.pdf</t>
+        </is>
+      </c>
+      <c r="L30" s="3" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="M30" s="3" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="N30" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="O30" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="P30" s="3" t="n"/>
+      <c r="Q30" s="3" t="n"/>
+      <c r="R30" s="3" t="n"/>
+      <c r="S30" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-16 13:17</t>
+        </is>
+      </c>
+      <c r="T30" s="3" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="80" customHeight="1">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>E-DA-029</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>database</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>recall</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="inlineStr">
+        <is>
+          <t>Database security and access control</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>explicit</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t>Which of the following references discusses an improved query performance technique using variant indexes?</t>
+        </is>
+      </c>
+      <c r="J31" s="2" t="inlineStr">
+        <is>
+          <t>The reference [O’Neil and Quass (1997)] discusses an improved query performance technique using variant indexes, as indicated in the context where it mentions "Improved Query Performance with Variant Indexes" in the proceedings of the ACM SIGMOD Conference on Management of Data.</t>
+        </is>
+      </c>
+      <c r="K31" s="2" t="inlineStr">
+        <is>
+          <t>source_8.pdf, source_31.pdf, source_7.pdf, source_36.pdf, source_49.pdf, source_13.pdf, source_14.pdf, source_18.pdf</t>
+        </is>
+      </c>
+      <c r="L31" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="M31" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N31" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="O31" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="P31" s="2" t="n"/>
+      <c r="Q31" s="2" t="n"/>
+      <c r="R31" s="2" t="n"/>
+      <c r="S31" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-16 13:18</t>
+        </is>
+      </c>
+      <c r="T31" s="2" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="80" customHeight="1">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>E-DA-030</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>database</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>recall</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="inlineStr">
+        <is>
+          <t>Data warehousing and OLAP</t>
+        </is>
+      </c>
+      <c r="F32" s="3" t="inlineStr">
+        <is>
+          <t>explicit</t>
+        </is>
+      </c>
+      <c r="G32" s="3" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H32" s="3" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="I32" s="3" t="inlineStr">
+        <is>
+          <t>What does the preface mention as making this book unique?</t>
+        </is>
+      </c>
+      <c r="J32" s="3" t="inlineStr">
+        <is>
+          <t>The preface mentions several features that make this book unique, including its clear distinction between basic material and advanced topics in Parts I and II, detailed descriptions of data warehouse architecture and schema, and coverage of data analysis operators such as drill-down, roll-up, and data cubes. Additionally, the book offers insights into relevant data mining problems and their solutions, distinguishing it from other texts in the field.</t>
+        </is>
+      </c>
+      <c r="K32" s="3" t="inlineStr">
+        <is>
+          <t>source_8.pdf, source_31.pdf, source_7.pdf, source_17.pdf, source_50.pdf, source_36.pdf, source_49.pdf, source_13.pdf, source_14.pdf, source_18.pdf</t>
+        </is>
+      </c>
+      <c r="L32" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="M32" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="N32" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="O32" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="P32" s="3" t="n"/>
+      <c r="Q32" s="3" t="n"/>
+      <c r="R32" s="3" t="n"/>
+      <c r="S32" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-16 13:18</t>
+        </is>
+      </c>
+      <c r="T32" s="3" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="80" customHeight="1">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>E-SO-031</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>software_engineering</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>recall</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="inlineStr">
+        <is>
+          <t>Software development lifecycle models</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>explicit</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>What are two key design issues that must be considered in distributed systems engineering, and briefly describe each?</t>
+        </is>
+      </c>
+      <c r="J33" s="2" t="inlineStr">
+        <is>
+          <t>Two key design issues in distributed systems engineering are transparency and openness. Transparency concerns the extent to which the distributed system appears as a single system to the user, determining when it is beneficial for users to be aware of the system's distributed nature. Openness involves whether the system should adhere to standard protocols supporting interoperability or utilize more specialized protocols that offer greater design flexibility but potentially reduce compatibility with other systems.</t>
+        </is>
+      </c>
+      <c r="K33" s="2" t="inlineStr">
+        <is>
+          <t>source_22.pdf</t>
+        </is>
+      </c>
+      <c r="L33" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="M33" s="2" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="N33" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="O33" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="P33" s="2" t="n"/>
+      <c r="Q33" s="2" t="n"/>
+      <c r="R33" s="2" t="n"/>
+      <c r="S33" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-16 13:37</t>
+        </is>
+      </c>
+      <c r="T33" s="2" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="80" customHeight="1">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>E-SO-032</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>software_engineering</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>recall</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="inlineStr">
+        <is>
+          <t>Agile methodology and requirements management</t>
+        </is>
+      </c>
+      <c r="F34" s="3" t="inlineStr">
+        <is>
+          <t>explicit</t>
+        </is>
+      </c>
+      <c r="G34" s="3" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H34" s="3" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="I34" s="3" t="inlineStr">
+        <is>
+          <t>According to the context, how do customers play a role in the agile development process?</t>
+        </is>
+      </c>
+      <c r="J34" s="3" t="inlineStr">
+        <is>
+          <t>Customers actively engage in the agile development process by proposing new and changed requirements after receiving working software at each iteration. This ongoing interaction ensures that the evolving needs of the customer are continuously integrated into the software development lifecycle, allowing for adaptive and responsive system development.</t>
+        </is>
+      </c>
+      <c r="K34" s="3" t="inlineStr">
+        <is>
+          <t>source_22.pdf, source_1.pdf, source_48.pdf, source_16.pdf, source_47.pdf, source_37.pdf, source_15.pdf, source_46.pdf, source_21.pdf, source_45.pdf, source_11.pdf</t>
+        </is>
+      </c>
+      <c r="L34" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="M34" s="3" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="N34" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="O34" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="P34" s="3" t="n"/>
+      <c r="Q34" s="3" t="n"/>
+      <c r="R34" s="3" t="n"/>
+      <c r="S34" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-16 13:38</t>
+        </is>
+      </c>
+      <c r="T34" s="3" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="80" customHeight="1">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>E-SO-033</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>software_engineering</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>recall</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="inlineStr">
+        <is>
+          <t>Verification and validation in software testing</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>explicit</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="I35" s="2" t="inlineStr">
+        <is>
+          <t>Which of the following best describes the difference between verification and testing as discussed in the context provided?</t>
+        </is>
+      </c>
+      <c r="J35" s="2" t="inlineStr">
+        <is>
+          <t>Verification and testing, as discussed in the context, differ in their objectives and scope. Verification focuses on ensuring that the product of development meets its specified requirements, often through static analysis or formal specification methods, whereas testing aims to discover faults by executing the software and observing its behavior under various conditions, including unit testing, integration testing, acceptance testing, and post-delivery maintenance.</t>
+        </is>
+      </c>
+      <c r="K35" s="2" t="inlineStr">
+        <is>
+          <t>source_22.pdf, source_1.pdf, source_48.pdf, source_46.pdf, source_21.pdf, source_11.pdf</t>
+        </is>
+      </c>
+      <c r="L35" s="2" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="M35" s="2" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="N35" s="2" t="n">
+        <v>1.67</v>
+      </c>
+      <c r="O35" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="P35" s="2" t="n"/>
+      <c r="Q35" s="2" t="n"/>
+      <c r="R35" s="2" t="n"/>
+      <c r="S35" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-16 13:40</t>
+        </is>
+      </c>
+      <c r="T35" s="2" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="80" customHeight="1">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>E-SO-034</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>software_engineering</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>recall</t>
+        </is>
+      </c>
+      <c r="E36" s="3" t="inlineStr">
+        <is>
+          <t>Unit testing and integration testing</t>
+        </is>
+      </c>
+      <c r="F36" s="3" t="inlineStr">
+        <is>
+          <t>explicit</t>
+        </is>
+      </c>
+      <c r="G36" s="3" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H36" s="3" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="I36" s="3" t="inlineStr">
+        <is>
+          <t>According to the Scrum methodology, which of the following best describes the iterative process involved in completing the backlog of tasks?</t>
+        </is>
+      </c>
+      <c r="J36" s="3" t="inlineStr">
+        <is>
+          <t>According to the Scrum methodology, the iterative process involves repeatedly conducting Requirements Sprints, where user stories are prioritized, daily meetings are held to discuss progress, and tasks are eventually reassigned as needed, until the backlog of tasks is completed. This cyclic approach ensures continuous refinement and delivery of new versions within fixed timeframes, promoting adaptive planning and frequent updates.</t>
+        </is>
+      </c>
+      <c r="K36" s="3" t="inlineStr">
+        <is>
+          <t>source_4.pdf, source_22.pdf, source_1.pdf, source_48.pdf, source_16.pdf, source_47.pdf, source_37.pdf, source_15.pdf, source_46.pdf, source_21.pdf, source_45.pdf, source_11.pdf</t>
+        </is>
+      </c>
+      <c r="L36" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="M36" s="3" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="N36" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="O36" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="P36" s="3" t="n"/>
+      <c r="Q36" s="3" t="n"/>
+      <c r="R36" s="3" t="n"/>
+      <c r="S36" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-16 13:41</t>
+        </is>
+      </c>
+      <c r="T36" s="3" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="80" customHeight="1">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>E-SO-035</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>software_engineering</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>recall</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="inlineStr">
+        <is>
+          <t>Test driven development</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>explicit</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="I37" s="2" t="inlineStr">
+        <is>
+          <t>What does test-driven development involve in terms of the sequence of activities between writing tests and developing code?</t>
+        </is>
+      </c>
+      <c r="J37" s="2" t="inlineStr">
+        <is>
+          <t>Test-driven development involves the programmer writing a failing test before developing the necessary code to pass that test, then refactoring the code as needed while ensuring the test continues to pass. This iterative process of writing tests followed by developing and refining the code ensures that each increment of functionality is thoroughly tested and meets the specified requirements.</t>
+        </is>
+      </c>
+      <c r="K37" s="2" t="inlineStr">
+        <is>
+          <t>source_4.pdf, source_22.pdf, source_1.pdf, source_48.pdf, source_47.pdf, source_37.pdf, source_21.pdf, source_45.pdf, source_11.pdf</t>
+        </is>
+      </c>
+      <c r="L37" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="M37" s="2" t="n">
+        <v>4.75</v>
+      </c>
+      <c r="N37" s="2" t="n">
+        <v>3.67</v>
+      </c>
+      <c r="O37" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="P37" s="2" t="n"/>
+      <c r="Q37" s="2" t="n"/>
+      <c r="R37" s="2" t="n"/>
+      <c r="S37" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-16 13:42</t>
+        </is>
+      </c>
+      <c r="T37" s="2" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="80" customHeight="1">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>E-SO-036</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>software_engineering</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>recall</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="inlineStr">
+        <is>
+          <t>Design patterns in object oriented programming</t>
+        </is>
+      </c>
+      <c r="F38" s="3" t="inlineStr">
+        <is>
+          <t>explicit</t>
+        </is>
+      </c>
+      <c r="G38" s="3" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H38" s="3" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="I38" s="3" t="inlineStr">
+        <is>
+          <t>What are the main objectives discussed in Chapter 7 of the course material regarding object-oriented design?</t>
+        </is>
+      </c>
+      <c r="J38" s="3" t="inlineStr">
+        <is>
+          <t>The main objectives discussed in Chapter 7 of the course material regarding object-oriented design are to introduce the fundamental activities involved in a general object-oriented design process and to highlight key implementation concerns such as reuse, configuration management, host-target development, and open-source development.</t>
+        </is>
+      </c>
+      <c r="K38" s="3" t="inlineStr">
+        <is>
+          <t>source_22.pdf, source_1.pdf, source_3.pdf, source_48.pdf, source_47.pdf, source_46.pdf, source_21.pdf, source_45.pdf, source_11.pdf</t>
+        </is>
+      </c>
+      <c r="L38" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="M38" s="3" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="N38" s="3" t="n">
+        <v>1.67</v>
+      </c>
+      <c r="O38" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="P38" s="3" t="n"/>
+      <c r="Q38" s="3" t="n"/>
+      <c r="R38" s="3" t="n"/>
+      <c r="S38" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-16 13:43</t>
+        </is>
+      </c>
+      <c r="T38" s="3" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="80" customHeight="1">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>E-SO-037</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>software_engineering</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>recall</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="inlineStr">
+        <is>
+          <t>Software architecture and modularity</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>explicit</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="I39" s="2" t="inlineStr">
+        <is>
+          <t>What is the importance of choosing the right architectural structure when designing a software system, according to the course material?</t>
+        </is>
+      </c>
+      <c r="J39" s="2" t="inlineStr">
+        <is>
+          <t>Choosing the right architectural structure is crucial as it directly influences the system's ability to meet specified requirements efficiently and effectively. The appropriate architectural structure ensures optimal decomposition of components and supports strategies for reuse and configuration management, thereby enhancing the overall quality and maintainability of the software system.</t>
+        </is>
+      </c>
+      <c r="K39" s="2" t="inlineStr">
+        <is>
+          <t>source_22.pdf, source_3.pdf, source_46.pdf, source_21.pdf, source_11.pdf</t>
+        </is>
+      </c>
+      <c r="L39" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="M39" s="2" t="n">
+        <v>3.75</v>
+      </c>
+      <c r="N39" s="2" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="O39" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="P39" s="2" t="n"/>
+      <c r="Q39" s="2" t="n"/>
+      <c r="R39" s="2" t="n"/>
+      <c r="S39" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-16 13:44</t>
+        </is>
+      </c>
+      <c r="T39" s="2" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="80" customHeight="1">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>E-SO-038</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>software_engineering</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>recall</t>
+        </is>
+      </c>
+      <c r="E40" s="3" t="inlineStr">
+        <is>
+          <t>Version control and configuration management</t>
+        </is>
+      </c>
+      <c r="F40" s="3" t="inlineStr">
+        <is>
+          <t>explicit</t>
+        </is>
+      </c>
+      <c r="G40" s="3" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H40" s="3" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="I40" s="3" t="inlineStr">
+        <is>
+          <t>What are the key processes involved in software change management according to Chapter 25?</t>
+        </is>
+      </c>
+      <c r="J40" s="3" t="inlineStr">
+        <is>
+          <t>The key processes involved in software change management according to Chapter 25 include change management itself, version management, and system building. These processes are interrelated, with version management providing essential functionality that supports system building and facilitating effective software change management.</t>
+        </is>
+      </c>
+      <c r="K40" s="3" t="inlineStr">
+        <is>
+          <t>source_22.pdf, source_1.pdf, source_3.pdf, source_47.pdf, source_46.pdf, source_21.pdf, source_45.pdf, source_11.pdf</t>
+        </is>
+      </c>
+      <c r="L40" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="M40" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="N40" s="3" t="n">
+        <v>1.67</v>
+      </c>
+      <c r="O40" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="P40" s="3" t="n"/>
+      <c r="Q40" s="3" t="n"/>
+      <c r="R40" s="3" t="n"/>
+      <c r="S40" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-16 13:45</t>
+        </is>
+      </c>
+      <c r="T40" s="3" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="80" customHeight="1">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>E-SO-039</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>software_engineering</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>recall</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>Code review and static analysis</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>explicit</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H41" s="2" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="I41" s="2" t="inlineStr">
+        <is>
+          <t>In which year was the paper "Using static analysis to find bugs" published?</t>
+        </is>
+      </c>
+      <c r="J41" s="2" t="inlineStr">
+        <is>
+          <t>The paper "Using static analysis to find bugs" was published in 2008, as indicated by the citation (N. Ayewah et al., IEEE Software, 25(5), Sept/Oct 2008.).</t>
+        </is>
+      </c>
+      <c r="K41" s="2" t="inlineStr">
+        <is>
+          <t>source_45.pdf, source_22.pdf</t>
+        </is>
+      </c>
+      <c r="L41" s="2" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="M41" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="N41" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="O41" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="P41" s="2" t="n"/>
+      <c r="Q41" s="2" t="n"/>
+      <c r="R41" s="2" t="n"/>
+      <c r="S41" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-16 13:46</t>
+        </is>
+      </c>
+      <c r="T41" s="2" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="80" customHeight="1">
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>E-SO-040</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>software_engineering</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>recall</t>
+        </is>
+      </c>
+      <c r="E42" s="3" t="inlineStr">
+        <is>
+          <t>Risk management in software projects</t>
+        </is>
+      </c>
+      <c r="F42" s="3" t="inlineStr">
+        <is>
+          <t>explicit</t>
+        </is>
+      </c>
+      <c r="G42" s="3" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H42" s="3" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="I42" s="3" t="inlineStr">
+        <is>
+          <t>What does the author, M. Ould, define as a risk in the context of project management, and how many categories of risk does he identify?</t>
+        </is>
+      </c>
+      <c r="J42" s="3" t="inlineStr">
+        <is>
+          <t>M. Ould defines a risk in the context of project management as something that one would prefer not to have happen, which could potentially affect the project schedule, the quality of the software being developed, or the organization itself. He identifies three related categories of risk: those that threaten the project, the software being developed, or the organization.</t>
+        </is>
+      </c>
+      <c r="K42" s="3" t="inlineStr">
+        <is>
+          <t>source_22.pdf, source_1.pdf, source_48.pdf, source_47.pdf, source_37.pdf, source_46.pdf, source_21.pdf, source_45.pdf, source_11.pdf</t>
+        </is>
+      </c>
+      <c r="L42" s="3" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="M42" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="N42" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="O42" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="P42" s="3" t="n"/>
+      <c r="Q42" s="3" t="n"/>
+      <c r="R42" s="3" t="n"/>
+      <c r="S42" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-16 13:48</t>
+        </is>
+      </c>
+      <c r="T42" s="3" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="80" customHeight="1">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>E-SO-041</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>software_engineering</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>recall</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="inlineStr">
+        <is>
+          <t>Requirements engineering and specification</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>explicit</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="I43" s="2" t="inlineStr">
+        <is>
+          <t>What does the manager assume about the relationship between the number of change requests and product usability and suitability?</t>
+        </is>
+      </c>
+      <c r="J43" s="2" t="inlineStr">
+        <is>
+          <t>The manager assumes that an increase in the number of change requests submitted by customers indicates lower product usability and suitability, suggesting that more changes are needed to improve the product's alignment with user needs and expectations.</t>
+        </is>
+      </c>
+      <c r="K43" s="2" t="inlineStr">
+        <is>
+          <t>source_22.pdf</t>
+        </is>
+      </c>
+      <c r="L43" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="M43" s="2" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="N43" s="2" t="n">
+        <v>3.67</v>
+      </c>
+      <c r="O43" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="P43" s="2" t="n"/>
+      <c r="Q43" s="2" t="n"/>
+      <c r="R43" s="2" t="n"/>
+      <c r="S43" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-16 13:49</t>
+        </is>
+      </c>
+      <c r="T43" s="2" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="80" customHeight="1">
+      <c r="A44" s="3" t="inlineStr">
+        <is>
+          <t>E-SO-042</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>software_engineering</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D44" s="3" t="inlineStr">
+        <is>
+          <t>recall</t>
+        </is>
+      </c>
+      <c r="E44" s="3" t="inlineStr">
+        <is>
+          <t>Software metrics and quality assurance</t>
+        </is>
+      </c>
+      <c r="F44" s="3" t="inlineStr">
+        <is>
+          <t>explicit</t>
+        </is>
+      </c>
+      <c r="G44" s="3" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H44" s="3" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="I44" s="3" t="inlineStr">
+        <is>
+          <t>According to the context provided, how should managers react to a very good programmer who produces software with a low number of defects but consistently ignores organizational quality standards?</t>
+        </is>
+      </c>
+      <c r="J44" s="3" t="inlineStr">
+        <is>
+          <t>Managers should address the contradiction between the programmer's technical excellence and disregard for organizational standards by first understanding the reasons behind this behavior. This may involve providing training on quality standards or aligning individual goals more closely with organizational objectives to ensure that high-quality standards are maintained while still valuing technical proficiency.</t>
+        </is>
+      </c>
+      <c r="K44" s="3" t="inlineStr">
+        <is>
+          <t>source_22.pdf</t>
+        </is>
+      </c>
+      <c r="L44" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="M44" s="3" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="N44" s="3" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="O44" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="P44" s="3" t="n"/>
+      <c r="Q44" s="3" t="n"/>
+      <c r="R44" s="3" t="n"/>
+      <c r="S44" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-16 13:51</t>
+        </is>
+      </c>
+      <c r="T44" s="3" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="80" customHeight="1">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>E-SO-043</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>software_engineering</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>recall</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>Refactoring and technical debt</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>explicit</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H45" s="2" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="I45" s="2" t="inlineStr">
+        <is>
+          <t>According to the context, which software tool, developed by Carlson, includes features that facilitate refactoring and make it easier to understand and modify the code?</t>
+        </is>
+      </c>
+      <c r="J45" s="2" t="inlineStr">
+        <is>
+          <t>According to Carlson's work, as detailed in "Eclipse Distilled" (Carlson, 2005), the Eclipse software tool includes features designed to facilitate refactoring, thereby simplifying the process of understanding and modifying code sections across the entire codebase.</t>
+        </is>
+      </c>
+      <c r="K45" s="2" t="inlineStr">
+        <is>
+          <t>source_22.pdf, source_1.pdf, source_48.pdf, source_47.pdf, source_37.pdf, source_46.pdf, source_21.pdf, source_45.pdf, source_11.pdf</t>
+        </is>
+      </c>
+      <c r="L45" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="M45" s="2" t="n">
+        <v>4.25</v>
+      </c>
+      <c r="N45" s="2" t="n">
+        <v>2.67</v>
+      </c>
+      <c r="O45" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="P45" s="2" t="n"/>
+      <c r="Q45" s="2" t="n"/>
+      <c r="R45" s="2" t="n"/>
+      <c r="S45" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-16 13:52</t>
+        </is>
+      </c>
+      <c r="T45" s="2" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="80" customHeight="1">
+      <c r="A46" s="3" t="inlineStr">
+        <is>
+          <t>E-SO-044</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>software_engineering</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D46" s="3" t="inlineStr">
+        <is>
+          <t>recall</t>
+        </is>
+      </c>
+      <c r="E46" s="3" t="inlineStr">
+        <is>
+          <t>Continuous integration and deployment</t>
+        </is>
+      </c>
+      <c r="F46" s="3" t="inlineStr">
+        <is>
+          <t>explicit</t>
+        </is>
+      </c>
+      <c r="G46" s="3" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H46" s="3" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="I46" s="3" t="inlineStr">
+        <is>
+          <t>What is a potential challenge when deploying a system that involves adapting it to diverse user environments, and how might this affect the system's de pendability?</t>
+        </is>
+      </c>
+      <c r="J46" s="3" t="inlineStr">
+        <is>
+          <t>Adapting a system to diverse user environments introduces significant challenges that can undermine its de pendability. Variations in user contexts necessitate extensive testing and customization, which may introduce unforeseen bugs or inconsistencies, thereby potentially compromising the system’s reliability and robustness.</t>
+        </is>
+      </c>
+      <c r="K46" s="3" t="inlineStr">
+        <is>
+          <t>source_21.pdf, source_22.pdf</t>
+        </is>
+      </c>
+      <c r="L46" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="M46" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="N46" s="3" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="O46" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="P46" s="3" t="n"/>
+      <c r="Q46" s="3" t="n"/>
+      <c r="R46" s="3" t="n"/>
+      <c r="S46" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-16 13:53</t>
+        </is>
+      </c>
+      <c r="T46" s="3" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="80" customHeight="1">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>E-SO-045</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>software_engineering</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="inlineStr">
+        <is>
+          <t>recall</t>
+        </is>
+      </c>
+      <c r="E47" s="2" t="inlineStr">
+        <is>
+          <t>Safety critical software testing</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>explicit</t>
+        </is>
+      </c>
+      <c r="G47" s="2" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H47" s="2" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="I47" s="2" t="inlineStr">
+        <is>
+          <t>According to Lutz (1993), what are the three classes of interface errors in complex systems?</t>
+        </is>
+      </c>
+      <c r="J47" s="2" t="inlineStr">
+        <is>
+          <t>According to Lutz (1993), interface errors in complex systems can be categorized into three classes: miscommunication errors, timing errors, and resource allocation errors.</t>
+        </is>
+      </c>
+      <c r="K47" s="2" t="inlineStr">
+        <is>
+          <t>source_22.pdf, source_46.pdf</t>
+        </is>
+      </c>
+      <c r="L47" s="2" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="M47" s="2" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="N47" s="2" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="O47" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="P47" s="2" t="n"/>
+      <c r="Q47" s="2" t="n"/>
+      <c r="R47" s="2" t="n"/>
+      <c r="S47" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-16 13:54</t>
+        </is>
+      </c>
+      <c r="T47" s="2" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="80" customHeight="1">
+      <c r="A48" s="7" t="inlineStr">
+        <is>
+          <t>E-OP-046</t>
+        </is>
+      </c>
+      <c r="B48" s="7" t="inlineStr">
+        <is>
+          <t>operating_systems</t>
+        </is>
+      </c>
+      <c r="C48" s="7" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D48" s="7" t="inlineStr">
+        <is>
+          <t>recall</t>
+        </is>
+      </c>
+      <c r="E48" s="7" t="inlineStr">
+        <is>
+          <t>Processes and threads</t>
+        </is>
+      </c>
+      <c r="F48" s="7" t="inlineStr">
+        <is>
+          <t>explicit</t>
+        </is>
+      </c>
+      <c r="G48" s="7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H48" s="7" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="I48" s="7" t="inlineStr">
+        <is>
+          <t>What happens if Process 1 is assigned Resource R1 and Process 2 is assigned Resource R2, and both processes need to access both resources to complete their functions? Describe the resulting situation using the terms introduced in the context.</t>
+        </is>
+      </c>
+      <c r="J48" s="7" t="inlineStr">
+        <is>
+          <t>If Process 1 is assigned Resource R1 and Process 2 is assigned Resource R2, and both processes require access to both resources to complete their functions, a deadlock can occur. Each process will wait indefinitely for the resource held by the other process, leading to a state where neither process can proceed, effectively deadlocking the system.</t>
+        </is>
+      </c>
+      <c r="K48" s="7" t="inlineStr">
+        <is>
+          <t>source_35.pdf, source_42.pdf, source_10.pdf, source_40.pdf, source_41.pdf, source_39.pdf, source_43.pdf, source_5.pdf, source_33.pdf</t>
+        </is>
+      </c>
+      <c r="L48" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="M48" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="N48" s="7" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="O48" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="P48" s="7" t="inlineStr"/>
+      <c r="Q48" s="7" t="inlineStr"/>
+      <c r="R48" s="7" t="inlineStr"/>
+      <c r="S48" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-16 14:01</t>
+        </is>
+      </c>
+      <c r="T48" s="7" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="80" customHeight="1">
+      <c r="A49" s="8" t="inlineStr">
+        <is>
+          <t>E-OP-047</t>
+        </is>
+      </c>
+      <c r="B49" s="8" t="inlineStr">
+        <is>
+          <t>operating_systems</t>
+        </is>
+      </c>
+      <c r="C49" s="8" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D49" s="8" t="inlineStr">
+        <is>
+          <t>recall</t>
+        </is>
+      </c>
+      <c r="E49" s="8" t="inlineStr">
+        <is>
+          <t>CPU scheduling algorithms</t>
+        </is>
+      </c>
+      <c r="F49" s="8" t="inlineStr">
+        <is>
+          <t>explicit</t>
+        </is>
+      </c>
+      <c r="G49" s="8" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H49" s="8" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="I49" s="8" t="inlineStr">
+        <is>
+          <t>Which of the following references provides a foundational understanding of CPU scheduling algorithms?</t>
+        </is>
+      </c>
+      <c r="J49" s="8" t="inlineStr">
+        <is>
+          <t>The foundational understanding of CPU scheduling algorithms is provided by Liu and Layland's seminal work, "Scheduling Algorithms for Multiprogramming in a Hard Real-time Environment," published in the Journal of the ACM in February 1973. This reference offers a critical analysis of scheduling techniques essential for managing processes in real-time systems.</t>
+        </is>
+      </c>
+      <c r="K49" s="8" t="inlineStr">
+        <is>
+          <t>source_5.pdf</t>
+        </is>
+      </c>
+      <c r="L49" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="M49" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="N49" s="8" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="O49" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="P49" s="8" t="inlineStr"/>
+      <c r="Q49" s="8" t="inlineStr"/>
+      <c r="R49" s="8" t="inlineStr"/>
+      <c r="S49" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-16 14:02</t>
+        </is>
+      </c>
+      <c r="T49" s="8" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="80" customHeight="1">
+      <c r="A50" s="7" t="inlineStr">
+        <is>
+          <t>E-OP-048</t>
+        </is>
+      </c>
+      <c r="B50" s="7" t="inlineStr">
+        <is>
+          <t>operating_systems</t>
+        </is>
+      </c>
+      <c r="C50" s="7" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D50" s="7" t="inlineStr">
+        <is>
+          <t>recall</t>
+        </is>
+      </c>
+      <c r="E50" s="7" t="inlineStr">
+        <is>
+          <t>Virtual memory and paging</t>
+        </is>
+      </c>
+      <c r="F50" s="7" t="inlineStr">
+        <is>
+          <t>explicit</t>
+        </is>
+      </c>
+      <c r="G50" s="7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H50" s="7" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="I50" s="7" t="inlineStr">
+        <is>
+          <t>What is the primary reason for keeping certain virtual locations in main memory during a block transfer when using paged virtual memory?</t>
+        </is>
+      </c>
+      <c r="J50" s="7" t="inlineStr">
+        <is>
+          <t>To ensure data integrity during a block transfer, certain virtual locations must remain in main memory when using paged virtual memory to prevent data loss. This is necessary because the transfer process is slow, and moving these critical segments out of main memory risks losing some of the data being transferred.</t>
+        </is>
+      </c>
+      <c r="K50" s="7" t="inlineStr">
+        <is>
+          <t>source_35.pdf, source_5.pdf, source_41.pdf, source_39.pdf, source_40.pdf</t>
+        </is>
+      </c>
+      <c r="L50" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="M50" s="7" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="N50" s="7" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="O50" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="P50" s="7" t="inlineStr"/>
+      <c r="Q50" s="7" t="inlineStr"/>
+      <c r="R50" s="7" t="inlineStr"/>
+      <c r="S50" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-16 14:02</t>
+        </is>
+      </c>
+      <c r="T50" s="7" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="80" customHeight="1">
+      <c r="A51" s="8" t="inlineStr">
+        <is>
+          <t>E-OP-049</t>
+        </is>
+      </c>
+      <c r="B51" s="8" t="inlineStr">
+        <is>
+          <t>operating_systems</t>
+        </is>
+      </c>
+      <c r="C51" s="8" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D51" s="8" t="inlineStr">
+        <is>
+          <t>recall</t>
+        </is>
+      </c>
+      <c r="E51" s="8" t="inlineStr">
+        <is>
+          <t>Deadlock detection and prevention</t>
+        </is>
+      </c>
+      <c r="F51" s="8" t="inlineStr">
+        <is>
+          <t>explicit</t>
+        </is>
+      </c>
+      <c r="G51" s="8" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H51" s="8" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="I51" s="8" t="inlineStr">
+        <is>
+          <t>What condition must be avoided in order to prevent deadlock according to the principles discussed in Chapter 6?</t>
+        </is>
+      </c>
+      <c r="J51" s="8" t="inlineStr">
+        <is>
+          <t>To prevent deadlock, the condition of circular wait must be avoided, as it is one of the necessary conditions for deadlock according to the principles discussed in Chapter 6. This involves ensuring that no set of processes can mutually hold at least one resource while waiting for another resource held by a process in the set, thus breaking the circular dependency that can lead to deadlock.</t>
+        </is>
+      </c>
+      <c r="K51" s="8" t="inlineStr">
+        <is>
+          <t>source_10.pdf, source_39.pdf, source_43.pdf, source_5.pdf, source_33.pdf</t>
+        </is>
+      </c>
+      <c r="L51" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="M51" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="N51" s="8" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="O51" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="P51" s="8" t="inlineStr"/>
+      <c r="Q51" s="8" t="inlineStr"/>
+      <c r="R51" s="8" t="inlineStr"/>
+      <c r="S51" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-16 14:03</t>
+        </is>
+      </c>
+      <c r="T51" s="8" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="80" customHeight="1">
+      <c r="A52" s="7" t="inlineStr">
+        <is>
+          <t>E-OP-050</t>
+        </is>
+      </c>
+      <c r="B52" s="7" t="inlineStr">
+        <is>
+          <t>operating_systems</t>
+        </is>
+      </c>
+      <c r="C52" s="7" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D52" s="7" t="inlineStr">
+        <is>
+          <t>recall</t>
+        </is>
+      </c>
+      <c r="E52" s="7" t="inlineStr">
+        <is>
+          <t>Banker algorithm and resource allocation</t>
+        </is>
+      </c>
+      <c r="F52" s="7" t="inlineStr">
+        <is>
+          <t>explicit</t>
+        </is>
+      </c>
+      <c r="G52" s="7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H52" s="7" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="I52" s="7" t="inlineStr">
+        <is>
+          <t>What does the formula `Need [i,j] = Max[i,j] - Allocation [i,j]` represent in the context of the banker's algorithm?</t>
+        </is>
+      </c>
+      <c r="J52" s="7" t="inlineStr">
+        <is>
+          <t>The formula `Need [i,j] = Max[i,j] - Allocation [i,j]` represents the calculation of the remaining resource requirements for each process with respect to each resource type under the banker's algorithm. Specifically, it determines how many additional instances of a given resource type a process needs to complete its task, based on the difference between its maximum required amount and the current allocation.</t>
+        </is>
+      </c>
+      <c r="K52" s="7" t="inlineStr">
+        <is>
+          <t>source_42.pdf, source_39.pdf, source_43.pdf, source_5.pdf, source_33.pdf</t>
+        </is>
+      </c>
+      <c r="L52" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="M52" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="N52" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="O52" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="P52" s="7" t="inlineStr"/>
+      <c r="Q52" s="7" t="inlineStr"/>
+      <c r="R52" s="7" t="inlineStr"/>
+      <c r="S52" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-16 14:03</t>
+        </is>
+      </c>
+      <c r="T52" s="7" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="80" customHeight="1">
+      <c r="A53" s="8" t="inlineStr">
+        <is>
+          <t>E-OP-051</t>
+        </is>
+      </c>
+      <c r="B53" s="8" t="inlineStr">
+        <is>
+          <t>operating_systems</t>
+        </is>
+      </c>
+      <c r="C53" s="8" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D53" s="8" t="inlineStr">
+        <is>
+          <t>recall</t>
+        </is>
+      </c>
+      <c r="E53" s="8" t="inlineStr">
+        <is>
+          <t>Memory management and segmentation</t>
+        </is>
+      </c>
+      <c r="F53" s="8" t="inlineStr">
+        <is>
+          <t>explicit</t>
+        </is>
+      </c>
+      <c r="G53" s="8" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H53" s="8" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="I53" s="8" t="inlineStr">
+        <is>
+          <t>What is the difference between segmentation and paging in the context of memory management?</t>
+        </is>
+      </c>
+      <c r="J53" s="8" t="inlineStr">
+        <is>
+          <t>Segmentation involves dividing a program into variable-length segments that reside in secondary memory, while paging entails dividing these segments into fixed-size pages that can be individually copied into main memory, allowing for more efficient memory management and addressing.</t>
+        </is>
+      </c>
+      <c r="K53" s="8" t="inlineStr">
+        <is>
+          <t>source_20.pdf, source_35.pdf, source_42.pdf, source_10.pdf, source_40.pdf, source_19.pdf, source_41.pdf, source_39.pdf, source_43.pdf, source_5.pdf, source_33.pdf</t>
+        </is>
+      </c>
+      <c r="L53" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="M53" s="8" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="N53" s="8" t="n">
+        <v>1.67</v>
+      </c>
+      <c r="O53" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="P53" s="8" t="inlineStr"/>
+      <c r="Q53" s="8" t="inlineStr"/>
+      <c r="R53" s="8" t="inlineStr"/>
+      <c r="S53" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-16 14:04</t>
+        </is>
+      </c>
+      <c r="T53" s="8" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="80" customHeight="1">
+      <c r="A54" s="7" t="inlineStr">
+        <is>
+          <t>E-OP-052</t>
+        </is>
+      </c>
+      <c r="B54" s="7" t="inlineStr">
+        <is>
+          <t>operating_systems</t>
+        </is>
+      </c>
+      <c r="C54" s="7" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D54" s="7" t="inlineStr">
+        <is>
+          <t>recall</t>
+        </is>
+      </c>
+      <c r="E54" s="7" t="inlineStr">
+        <is>
+          <t>File systems and directory structures</t>
+        </is>
+      </c>
+      <c r="F54" s="7" t="inlineStr">
+        <is>
+          <t>explicit</t>
+        </is>
+      </c>
+      <c r="G54" s="7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H54" s="7" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="I54" s="7" t="inlineStr">
+        <is>
+          <t>What is the primary advantage of an indexed sequential file over a sequential file?</t>
+        </is>
+      </c>
+      <c r="J54" s="7" t="inlineStr">
+        <is>
+          <t>An indexed sequential file offers faster search capabilities compared to a sequential file by maintaining an index, allowing for direct access to records based on key values, whereas a sequential file requires linear search through all records to locate a specific entry.</t>
+        </is>
+      </c>
+      <c r="K54" s="7" t="inlineStr">
+        <is>
+          <t>source_20.pdf, source_35.pdf, source_40.pdf, source_41.pdf, source_39.pdf, source_43.pdf, source_5.pdf, source_33.pdf</t>
+        </is>
+      </c>
+      <c r="L54" s="7" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="M54" s="7" t="n">
+        <v>4.75</v>
+      </c>
+      <c r="N54" s="7" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="O54" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="P54" s="7" t="inlineStr"/>
+      <c r="Q54" s="7" t="inlineStr"/>
+      <c r="R54" s="7" t="inlineStr"/>
+      <c r="S54" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-16 14:05</t>
+        </is>
+      </c>
+      <c r="T54" s="7" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="80" customHeight="1">
+      <c r="A55" s="8" t="inlineStr">
+        <is>
+          <t>E-OP-053</t>
+        </is>
+      </c>
+      <c r="B55" s="8" t="inlineStr">
+        <is>
+          <t>operating_systems</t>
+        </is>
+      </c>
+      <c r="C55" s="8" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D55" s="8" t="inlineStr">
+        <is>
+          <t>recall</t>
+        </is>
+      </c>
+      <c r="E55" s="8" t="inlineStr">
+        <is>
+          <t>Interprocess communication</t>
+        </is>
+      </c>
+      <c r="F55" s="8" t="inlineStr">
+        <is>
+          <t>explicit</t>
+        </is>
+      </c>
+      <c r="G55" s="8" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H55" s="8" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="I55" s="8" t="inlineStr">
+        <is>
+          <t>What does the operating system manage on behalf of its users regarding secondary memory and I/O devices?</t>
+        </is>
+      </c>
+      <c r="J55" s="8" t="inlineStr">
+        <is>
+          <t>The operating system manages secondary memory and I/O devices on behalf of its users by controlling their access and ensuring efficient data transfer, thereby providing a stable and secure environment for user operations.</t>
+        </is>
+      </c>
+      <c r="K55" s="8" t="inlineStr">
+        <is>
+          <t>source_5.pdf, source_42.pdf, source_19.pdf, source_39.pdf, source_40.pdf</t>
+        </is>
+      </c>
+      <c r="L55" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="M55" s="8" t="n">
+        <v>4</v>
+      </c>
+      <c r="N55" s="8" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="O55" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="P55" s="8" t="inlineStr"/>
+      <c r="Q55" s="8" t="inlineStr"/>
+      <c r="R55" s="8" t="inlineStr"/>
+      <c r="S55" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-16 14:06</t>
+        </is>
+      </c>
+      <c r="T55" s="8" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="80" customHeight="1">
+      <c r="A56" s="7" t="inlineStr">
+        <is>
+          <t>E-OP-054</t>
+        </is>
+      </c>
+      <c r="B56" s="7" t="inlineStr">
+        <is>
+          <t>operating_systems</t>
+        </is>
+      </c>
+      <c r="C56" s="7" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D56" s="7" t="inlineStr">
+        <is>
+          <t>recall</t>
+        </is>
+      </c>
+      <c r="E56" s="7" t="inlineStr">
+        <is>
+          <t>Semaphores and mutual exclusion</t>
+        </is>
+      </c>
+      <c r="F56" s="7" t="inlineStr">
+        <is>
+          <t>explicit</t>
+        </is>
+      </c>
+      <c r="G56" s="7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H56" s="7" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="I56" s="7" t="inlineStr">
+        <is>
+          <t>Which of the following concepts does NOT illustrate the operation of mutual exclusion?</t>
+        </is>
+      </c>
+      <c r="J56" s="7" t="inlineStr">
+        <is>
+          <t>The Eisenberg-McGuire algorithm illustrates a software approach to mutual exclusion, whereas semaphores, reader-writer, and message passing problems pertain to the operation of mutual exclusion. Therefore, the concept that does not illustrate the operation of mutual exclusion is the Eisenberg-McGuire algorithm.</t>
+        </is>
+      </c>
+      <c r="K56" s="7" t="inlineStr">
+        <is>
+          <t>source_20.pdf, source_35.pdf, source_10.pdf, source_42.pdf, source_40.pdf, source_41.pdf, source_39.pdf, source_43.pdf, source_5.pdf, source_33.pdf</t>
+        </is>
+      </c>
+      <c r="L56" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="M56" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="N56" s="7" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="O56" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="P56" s="7" t="inlineStr"/>
+      <c r="Q56" s="7" t="inlineStr"/>
+      <c r="R56" s="7" t="inlineStr"/>
+      <c r="S56" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-16 14:06</t>
+        </is>
+      </c>
+      <c r="T56" s="7" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="80" customHeight="1">
+      <c r="A57" s="8" t="inlineStr">
+        <is>
+          <t>E-OP-055</t>
+        </is>
+      </c>
+      <c r="B57" s="8" t="inlineStr">
+        <is>
+          <t>operating_systems</t>
+        </is>
+      </c>
+      <c r="C57" s="8" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D57" s="8" t="inlineStr">
+        <is>
+          <t>recall</t>
+        </is>
+      </c>
+      <c r="E57" s="8" t="inlineStr">
+        <is>
+          <t>Disk scheduling algorithms</t>
+        </is>
+      </c>
+      <c r="F57" s="8" t="inlineStr">
+        <is>
+          <t>explicit</t>
+        </is>
+      </c>
+      <c r="G57" s="8" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H57" s="8" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="I57" s="8" t="inlineStr">
+        <is>
+          <t>Which book provides a detailed discussion on disk scheduling algorithms?</t>
+        </is>
+      </c>
+      <c r="J57" s="8" t="inlineStr">
+        <is>
+          <t>Selzer et al.'s "Disk Scheduling Revisited" from the Proceedings of the USENIX Winter Technical Conference in 1990 offers a detailed discussion on disk scheduling algorithms.</t>
+        </is>
+      </c>
+      <c r="K57" s="8" t="inlineStr">
+        <is>
+          <t>source_20.pdf, source_35.pdf, source_5.pdf, source_10.pdf, source_41.pdf, source_39.pdf, source_40.pdf</t>
+        </is>
+      </c>
+      <c r="L57" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="M57" s="8" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="N57" s="8" t="n">
+        <v>1.67</v>
+      </c>
+      <c r="O57" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="P57" s="8" t="inlineStr"/>
+      <c r="Q57" s="8" t="inlineStr"/>
+      <c r="R57" s="8" t="inlineStr"/>
+      <c r="S57" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-16 14:07</t>
+        </is>
+      </c>
+      <c r="T57" s="8" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="80" customHeight="1">
+      <c r="A58" s="7" t="inlineStr">
+        <is>
+          <t>E-OP-056</t>
+        </is>
+      </c>
+      <c r="B58" s="7" t="inlineStr">
+        <is>
+          <t>operating_systems</t>
+        </is>
+      </c>
+      <c r="C58" s="7" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D58" s="7" t="inlineStr">
+        <is>
+          <t>recall</t>
+        </is>
+      </c>
+      <c r="E58" s="7" t="inlineStr">
+        <is>
+          <t>Page replacement algorithms</t>
+        </is>
+      </c>
+      <c r="F58" s="7" t="inlineStr">
+        <is>
+          <t>explicit</t>
+        </is>
+      </c>
+      <c r="G58" s="7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H58" s="7" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="I58" s="7" t="inlineStr">
+        <is>
+          <t>Which of the following best describes why the FIFO page replacement algorithm may not be optimal in a multiprogramming environment?</t>
+        </is>
+      </c>
+      <c r="J58" s="7" t="inlineStr">
+        <is>
+          <t>The FIFO page replacement algorithm may not be optimal in a multiprogramming environment because it tends to replace pages that have been in memory for the longest period, which often includes frequently accessed pages that remain in use throughout the program's execution. This results in unnecessary page faults for frequently used pages, leading to poor performance compared to more sophisticated algorithms like LRU, which aims to keep recently used pages in memory.</t>
+        </is>
+      </c>
+      <c r="K58" s="7" t="inlineStr">
+        <is>
+          <t>source_20.pdf, source_35.pdf, source_5.pdf, source_42.pdf, source_10.pdf, source_41.pdf, source_39.pdf, source_40.pdf, source_33.pdf</t>
+        </is>
+      </c>
+      <c r="L58" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="M58" s="7" t="n">
+        <v>2.75</v>
+      </c>
+      <c r="N58" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="O58" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="P58" s="7" t="inlineStr"/>
+      <c r="Q58" s="7" t="inlineStr"/>
+      <c r="R58" s="7" t="inlineStr"/>
+      <c r="S58" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-16 14:07</t>
+        </is>
+      </c>
+      <c r="T58" s="7" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="80" customHeight="1">
+      <c r="A59" s="8" t="inlineStr">
+        <is>
+          <t>E-OP-057</t>
+        </is>
+      </c>
+      <c r="B59" s="8" t="inlineStr">
+        <is>
+          <t>operating_systems</t>
+        </is>
+      </c>
+      <c r="C59" s="8" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D59" s="8" t="inlineStr">
+        <is>
+          <t>recall</t>
+        </is>
+      </c>
+      <c r="E59" s="8" t="inlineStr">
+        <is>
+          <t>System calls and kernel mode</t>
+        </is>
+      </c>
+      <c r="F59" s="8" t="inlineStr">
+        <is>
+          <t>explicit</t>
+        </is>
+      </c>
+      <c r="G59" s="8" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H59" s="8" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="I59" s="8" t="inlineStr">
+        <is>
+          <t>What does the term "exception" refer to in the context of operating systems, and provide an example of an illegal program action that would trigger an exception?</t>
+        </is>
+      </c>
+      <c r="J59" s="8" t="inlineStr">
+        <is>
+          <t>In the context of operating systems, an exception refers to an illegal program action that generates an interrupt. An example of such an illegal action is attempting to access memory for a PTE that is not present, which would trigger an exception.</t>
+        </is>
+      </c>
+      <c r="K59" s="8" t="inlineStr">
+        <is>
+          <t>source_35.pdf, source_5.pdf, source_41.pdf, source_39.pdf, source_40.pdf</t>
+        </is>
+      </c>
+      <c r="L59" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="M59" s="8" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="N59" s="8" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="O59" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="P59" s="8" t="inlineStr"/>
+      <c r="Q59" s="8" t="inlineStr"/>
+      <c r="R59" s="8" t="inlineStr"/>
+      <c r="S59" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-16 14:08</t>
+        </is>
+      </c>
+      <c r="T59" s="8" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="80" customHeight="1">
+      <c r="A60" s="7" t="inlineStr">
+        <is>
+          <t>E-OP-058</t>
+        </is>
+      </c>
+      <c r="B60" s="7" t="inlineStr">
+        <is>
+          <t>operating_systems</t>
+        </is>
+      </c>
+      <c r="C60" s="7" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D60" s="7" t="inlineStr">
+        <is>
+          <t>recall</t>
+        </is>
+      </c>
+      <c r="E60" s="7" t="inlineStr">
+        <is>
+          <t>Context switching and process states</t>
+        </is>
+      </c>
+      <c r="F60" s="7" t="inlineStr">
+        <is>
+          <t>explicit</t>
+        </is>
+      </c>
+      <c r="G60" s="7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H60" s="7" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="I60" s="7" t="inlineStr">
+        <is>
+          <t>What is the maximum response time allowed for conversational interaction according to Table 9.7?</t>
+        </is>
+      </c>
+      <c r="J60" s="7" t="inlineStr">
+        <is>
+          <t>According to Table 9.7, the maximum response time allowed for conversational interaction is less than 15 seconds, as any response time greater than 15 seconds would rule out such interaction.</t>
+        </is>
+      </c>
+      <c r="K60" s="7" t="inlineStr">
+        <is>
+          <t>source_35.pdf, source_5.pdf, source_39.pdf, source_40.pdf, source_33.pdf</t>
+        </is>
+      </c>
+      <c r="L60" s="7" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="M60" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="N60" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="O60" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="P60" s="7" t="inlineStr"/>
+      <c r="Q60" s="7" t="inlineStr"/>
+      <c r="R60" s="7" t="inlineStr"/>
+      <c r="S60" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-16 14:09</t>
+        </is>
+      </c>
+      <c r="T60" s="7" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="80" customHeight="1">
+      <c r="A61" s="8" t="inlineStr">
+        <is>
+          <t>E-OP-059</t>
+        </is>
+      </c>
+      <c r="B61" s="8" t="inlineStr">
+        <is>
+          <t>operating_systems</t>
+        </is>
+      </c>
+      <c r="C61" s="8" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D61" s="8" t="inlineStr">
+        <is>
+          <t>recall</t>
+        </is>
+      </c>
+      <c r="E61" s="8" t="inlineStr">
+        <is>
+          <t>Real time operating systems</t>
+        </is>
+      </c>
+      <c r="F61" s="8" t="inlineStr">
+        <is>
+          <t>explicit</t>
+        </is>
+      </c>
+      <c r="G61" s="8" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H61" s="8" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="I61" s="8" t="inlineStr">
+        <is>
+          <t>Which two example systems are discussed in the chapter on embedded operating systems?</t>
+        </is>
+      </c>
+      <c r="J61" s="8" t="inlineStr">
+        <is>
+          <t>The chapter on embedded operating systems discusses two example systems: eCOS and TinyOS.</t>
+        </is>
+      </c>
+      <c r="K61" s="8" t="inlineStr">
+        <is>
+          <t>source_41.pdf, source_5.pdf</t>
+        </is>
+      </c>
+      <c r="L61" s="8" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="M61" s="8" t="n">
+        <v>2</v>
+      </c>
+      <c r="N61" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="O61" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="P61" s="8" t="inlineStr"/>
+      <c r="Q61" s="8" t="inlineStr"/>
+      <c r="R61" s="8" t="inlineStr"/>
+      <c r="S61" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-16 14:09</t>
+        </is>
+      </c>
+      <c r="T61" s="8" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="80" customHeight="1">
+      <c r="A62" s="7" t="inlineStr">
+        <is>
+          <t>E-OP-060</t>
+        </is>
+      </c>
+      <c r="B62" s="7" t="inlineStr">
+        <is>
+          <t>operating_systems</t>
+        </is>
+      </c>
+      <c r="C62" s="7" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D62" s="7" t="inlineStr">
+        <is>
+          <t>recall</t>
+        </is>
+      </c>
+      <c r="E62" s="7" t="inlineStr">
+        <is>
+          <t>Input output management</t>
+        </is>
+      </c>
+      <c r="F62" s="7" t="inlineStr">
+        <is>
+          <t>explicit</t>
+        </is>
+      </c>
+      <c r="G62" s="7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H62" s="7" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="I62" s="7" t="inlineStr">
+        <is>
+          <t>What is the role of an operating system in managing input/output operations, and how does it relate to the computer system hardware?</t>
+        </is>
+      </c>
+      <c r="J62" s="7" t="inlineStr">
+        <is>
+          <t>The operating system plays a crucial role in managing input/output operations by acting as an intermediary between application programs and the underlying hardware. It ensures efficient communication and resource allocation between software requests and physical hardware components, thereby facilitating the seamless interaction between user-level processes and the I/O devices.</t>
+        </is>
+      </c>
+      <c r="K62" s="7" t="inlineStr">
+        <is>
+          <t>source_35.pdf, source_10.pdf, source_40.pdf, source_41.pdf, source_39.pdf, source_5.pdf, source_33.pdf</t>
+        </is>
+      </c>
+      <c r="L62" s="7" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="M62" s="7" t="n">
+        <v>4.75</v>
+      </c>
+      <c r="N62" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="O62" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="P62" s="7" t="inlineStr"/>
+      <c r="Q62" s="7" t="inlineStr"/>
+      <c r="R62" s="7" t="inlineStr"/>
+      <c r="S62" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-16 14:10</t>
+        </is>
+      </c>
+      <c r="T62" s="7" t="inlineStr">
         <is>
           <t>done</t>
         </is>

</xml_diff>

<commit_message>
complete easy category 75 questions generated across all 5 domains refs #refs 91
</commit_message>
<xml_diff>
--- a/dataset/outputs/P000233DS_Question_Dataset.xlsx
+++ b/dataset/outputs/P000233DS_Question_Dataset.xlsx
@@ -540,7 +540,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T62"/>
+  <dimension ref="A1:T77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5" outlineLevelCol="0"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -5638,6 +5638,1248 @@
         </is>
       </c>
     </row>
+    <row r="63" ht="80" customHeight="1">
+      <c r="A63" s="8" t="inlineStr">
+        <is>
+          <t>E-CO-061</t>
+        </is>
+      </c>
+      <c r="B63" s="8" t="inlineStr">
+        <is>
+          <t>computer_architecture</t>
+        </is>
+      </c>
+      <c r="C63" s="8" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D63" s="8" t="inlineStr">
+        <is>
+          <t>recall</t>
+        </is>
+      </c>
+      <c r="E63" s="8" t="inlineStr">
+        <is>
+          <t>Instruction pipelining</t>
+        </is>
+      </c>
+      <c r="F63" s="8" t="inlineStr">
+        <is>
+          <t>explicit</t>
+        </is>
+      </c>
+      <c r="G63" s="8" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H63" s="8" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="I63" s="8" t="inlineStr">
+        <is>
+          <t>What does the "C" in RV32IC stand for, and what is its primary purpose?</t>
+        </is>
+      </c>
+      <c r="J63" s="8" t="inlineStr">
+        <is>
+          <t>The "C" in RV32IC stands for "compressed," indicating that this variant of the RISC-V instruction set includes 16-bit instructions for common operations, particularly those involving small intermediate values and ALU operations where the source and destination registers are identical. This compression allows for more efficient encoding of frequently used instructions, thereby improving code density and potentially enhancing performance in embedded systems and other applications where instruction cache utilization is critical.</t>
+        </is>
+      </c>
+      <c r="K63" s="8" t="inlineStr">
+        <is>
+          <t>source_12.pdf</t>
+        </is>
+      </c>
+      <c r="L63" s="8" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="M63" s="8" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="N63" s="8" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="O63" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="P63" s="8" t="inlineStr"/>
+      <c r="Q63" s="8" t="inlineStr"/>
+      <c r="R63" s="8" t="inlineStr"/>
+      <c r="S63" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-16 14:26</t>
+        </is>
+      </c>
+      <c r="T63" s="8" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="80" customHeight="1">
+      <c r="A64" s="7" t="inlineStr">
+        <is>
+          <t>E-CO-062</t>
+        </is>
+      </c>
+      <c r="B64" s="7" t="inlineStr">
+        <is>
+          <t>computer_architecture</t>
+        </is>
+      </c>
+      <c r="C64" s="7" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D64" s="7" t="inlineStr">
+        <is>
+          <t>recall</t>
+        </is>
+      </c>
+      <c r="E64" s="7" t="inlineStr">
+        <is>
+          <t>Cache memory hierarchy</t>
+        </is>
+      </c>
+      <c r="F64" s="7" t="inlineStr">
+        <is>
+          <t>explicit</t>
+        </is>
+      </c>
+      <c r="G64" s="7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H64" s="7" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="I64" s="7" t="inlineStr">
+        <is>
+          <t>Explain the conditions under which inclusion is maintained in a two-level cache hierarchy where L1 is closer to the processor.</t>
+        </is>
+      </c>
+      <c r="J64" s="7" t="inlineStr">
+        <is>
+          <t>Inclusion is maintained in a two-level cache hierarchy where L1 is closer to the processor, provided that L2 has at least as much associativity as L1, both caches employ LRU replacement policy, and they share the same block sizes. This ensures that any data present in the L1 cache will also be found in the L2 cache without requiring additional actions to maintain this property.</t>
+        </is>
+      </c>
+      <c r="K64" s="7" t="inlineStr">
+        <is>
+          <t>source_44.pdf, source_29.pdf, source_30.pdf, source_6.pdf, source_23.pdf, source_24.pdf, source_38.pdf, source_25.pdf, source_28.pdf, source_9.pdf, source_26.pdf, source_12.pdf</t>
+        </is>
+      </c>
+      <c r="L64" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="M64" s="7" t="n">
+        <v>4.25</v>
+      </c>
+      <c r="N64" s="7" t="n">
+        <v>1.67</v>
+      </c>
+      <c r="O64" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="P64" s="7" t="inlineStr"/>
+      <c r="Q64" s="7" t="inlineStr"/>
+      <c r="R64" s="7" t="inlineStr"/>
+      <c r="S64" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-16 14:27</t>
+        </is>
+      </c>
+      <c r="T64" s="7" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="80" customHeight="1">
+      <c r="A65" s="8" t="inlineStr">
+        <is>
+          <t>E-CO-063</t>
+        </is>
+      </c>
+      <c r="B65" s="8" t="inlineStr">
+        <is>
+          <t>computer_architecture</t>
+        </is>
+      </c>
+      <c r="C65" s="8" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D65" s="8" t="inlineStr">
+        <is>
+          <t>recall</t>
+        </is>
+      </c>
+      <c r="E65" s="8" t="inlineStr">
+        <is>
+          <t>Pipeline hazards and resolution techniques</t>
+        </is>
+      </c>
+      <c r="F65" s="8" t="inlineStr">
+        <is>
+          <t>explicit</t>
+        </is>
+      </c>
+      <c r="G65" s="8" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H65" s="8" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="I65" s="8" t="inlineStr">
+        <is>
+          <t>What is the "major hurdle" of pipelining mentioned in the context, and why is it particularly challenging for processors with longer pipelines that issue multiple instructions per clock cycle?</t>
+        </is>
+      </c>
+      <c r="J65" s="8" t="inlineStr">
+        <is>
+          <t>The major hurdle of pipelining, as mentioned in the context, refers to pipeline hazards. These hazards become particularly challenging for processors with longer pipelines that issue multiple instructions per clock cycle because the complex interactions between instructions can lead to stalls and misalignments, thereby reducing the efficiency gains intended by pipelining.</t>
+        </is>
+      </c>
+      <c r="K65" s="8" t="inlineStr">
+        <is>
+          <t>source_29.pdf, source_32.pdf, source_6.pdf, source_30.pdf, source_23.pdf, source_24.pdf, source_38.pdf, source_25.pdf, source_27.pdf, source_28.pdf, source_9.pdf, source_26.pdf, source_12.pdf</t>
+        </is>
+      </c>
+      <c r="L65" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="M65" s="8" t="n">
+        <v>4.75</v>
+      </c>
+      <c r="N65" s="8" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="O65" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="P65" s="8" t="inlineStr"/>
+      <c r="Q65" s="8" t="inlineStr"/>
+      <c r="R65" s="8" t="inlineStr"/>
+      <c r="S65" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-16 14:27</t>
+        </is>
+      </c>
+      <c r="T65" s="8" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="80" customHeight="1">
+      <c r="A66" s="7" t="inlineStr">
+        <is>
+          <t>E-CO-064</t>
+        </is>
+      </c>
+      <c r="B66" s="7" t="inlineStr">
+        <is>
+          <t>computer_architecture</t>
+        </is>
+      </c>
+      <c r="C66" s="7" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D66" s="7" t="inlineStr">
+        <is>
+          <t>recall</t>
+        </is>
+      </c>
+      <c r="E66" s="7" t="inlineStr">
+        <is>
+          <t>Memory hierarchy and locality</t>
+        </is>
+      </c>
+      <c r="F66" s="7" t="inlineStr">
+        <is>
+          <t>explicit</t>
+        </is>
+      </c>
+      <c r="G66" s="7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H66" s="7" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="I66" s="7" t="inlineStr">
+        <is>
+          <t>What are the key components discussed in the context of the design of memory hierarchies in Chapters 2.5 and 2.6 of the course material?</t>
+        </is>
+      </c>
+      <c r="J66" s="7" t="inlineStr">
+        <is>
+          <t>The key components discussed in the context of the design of memory hierarchies in Chapters 2.5 and 2.6 include the role of cache, technology advancements, and specific implementations such as those in the ARM Cortex-A53 and Intel Core i7 6700 processors. These chapters explore how these elements contribute to efficient memory management and access in modern computing architectures.</t>
+        </is>
+      </c>
+      <c r="K66" s="7" t="inlineStr">
+        <is>
+          <t>source_44.pdf, source_29.pdf, source_32.pdf, source_30.pdf, source_6.pdf, source_23.pdf, source_24.pdf, source_38.pdf, source_27.pdf, source_25.pdf, source_28.pdf, source_9.pdf, source_26.pdf, source_12.pdf</t>
+        </is>
+      </c>
+      <c r="L66" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="M66" s="7" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="N66" s="7" t="n">
+        <v>1.67</v>
+      </c>
+      <c r="O66" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="P66" s="7" t="inlineStr"/>
+      <c r="Q66" s="7" t="inlineStr"/>
+      <c r="R66" s="7" t="inlineStr"/>
+      <c r="S66" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-16 14:28</t>
+        </is>
+      </c>
+      <c r="T66" s="7" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="80" customHeight="1">
+      <c r="A67" s="8" t="inlineStr">
+        <is>
+          <t>E-CO-065</t>
+        </is>
+      </c>
+      <c r="B67" s="8" t="inlineStr">
+        <is>
+          <t>computer_architecture</t>
+        </is>
+      </c>
+      <c r="C67" s="8" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D67" s="8" t="inlineStr">
+        <is>
+          <t>recall</t>
+        </is>
+      </c>
+      <c r="E67" s="8" t="inlineStr">
+        <is>
+          <t>Instruction set architecture</t>
+        </is>
+      </c>
+      <c r="F67" s="8" t="inlineStr">
+        <is>
+          <t>explicit</t>
+        </is>
+      </c>
+      <c r="G67" s="8" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H67" s="8" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="I67" s="8" t="inlineStr">
+        <is>
+          <t>Which of the following architectures is mentioned in Appendix K as an example of a many RISC architecture?</t>
+        </is>
+      </c>
+      <c r="J67" s="8" t="inlineStr">
+        <is>
+          <t>ARM is mentioned in Appendix K as an example of a many RISC architecture.</t>
+        </is>
+      </c>
+      <c r="K67" s="8" t="inlineStr">
+        <is>
+          <t>source_30.pdf, source_23.pdf, source_24.pdf, source_38.pdf, source_9.pdf, source_12.pdf</t>
+        </is>
+      </c>
+      <c r="L67" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="M67" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="N67" s="8" t="n">
+        <v>1.67</v>
+      </c>
+      <c r="O67" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="P67" s="8" t="inlineStr"/>
+      <c r="Q67" s="8" t="inlineStr"/>
+      <c r="R67" s="8" t="inlineStr"/>
+      <c r="S67" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-16 14:28</t>
+        </is>
+      </c>
+      <c r="T67" s="8" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="80" customHeight="1">
+      <c r="A68" s="7" t="inlineStr">
+        <is>
+          <t>E-CO-066</t>
+        </is>
+      </c>
+      <c r="B68" s="7" t="inlineStr">
+        <is>
+          <t>computer_architecture</t>
+        </is>
+      </c>
+      <c r="C68" s="7" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D68" s="7" t="inlineStr">
+        <is>
+          <t>recall</t>
+        </is>
+      </c>
+      <c r="E68" s="7" t="inlineStr">
+        <is>
+          <t>Superscalar and out of order execution</t>
+        </is>
+      </c>
+      <c r="F68" s="7" t="inlineStr">
+        <is>
+          <t>explicit</t>
+        </is>
+      </c>
+      <c r="G68" s="7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H68" s="7" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="I68" s="7" t="inlineStr">
+        <is>
+          <t>Rewrite the following assembly code using a conditional move (CMOV) instruction to eliminate the branch at instruction 2:
+Original Code:
+1. ADD R1, R2, R3
+2. JZ R4, Label1
+3. SUB R5, R6, R7
+4. Label1: ...</t>
+        </is>
+      </c>
+      <c r="J68" s="7" t="inlineStr">
+        <is>
+          <t>To eliminate the branch at instruction 2, we can utilize the conditional move (CMOV) instruction to replace the jump instruction. The original jump condition can be translated into a CMOV instruction that sets R4 to zero if the condition is met, thereby effectively removing the need for the branch. The rewritten code would look like this:
+```
+1. ADD R1, R2, R3
+2. CMOVEQZ R4, #0, R4  # If R2 == 0, then R4 = 0; otherwise, R4 remains unchanged.
+3. SUB R5, R6, R7
+4. Label1: ...
+```
+This approach leverages the CMOV instruction to conditionally set R4 to zero based on the zero flag, thus eliminating the branch at instruction 2 while preserving the flow control logic.</t>
+        </is>
+      </c>
+      <c r="K68" s="7" t="inlineStr">
+        <is>
+          <t>source_29.pdf, source_32.pdf, source_30.pdf, source_6.pdf, source_23.pdf, source_38.pdf, source_25.pdf, source_27.pdf, source_28.pdf, source_9.pdf, source_12.pdf</t>
+        </is>
+      </c>
+      <c r="L68" s="7" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="M68" s="7" t="n">
+        <v>4</v>
+      </c>
+      <c r="N68" s="7" t="n">
+        <v>1.67</v>
+      </c>
+      <c r="O68" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="P68" s="7" t="inlineStr"/>
+      <c r="Q68" s="7" t="inlineStr"/>
+      <c r="R68" s="7" t="inlineStr"/>
+      <c r="S68" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-16 14:30</t>
+        </is>
+      </c>
+      <c r="T68" s="7" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="80" customHeight="1">
+      <c r="A69" s="8" t="inlineStr">
+        <is>
+          <t>E-CO-067</t>
+        </is>
+      </c>
+      <c r="B69" s="8" t="inlineStr">
+        <is>
+          <t>computer_architecture</t>
+        </is>
+      </c>
+      <c r="C69" s="8" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D69" s="8" t="inlineStr">
+        <is>
+          <t>recall</t>
+        </is>
+      </c>
+      <c r="E69" s="8" t="inlineStr">
+        <is>
+          <t>Branch prediction</t>
+        </is>
+      </c>
+      <c r="F69" s="8" t="inlineStr">
+        <is>
+          <t>explicit</t>
+        </is>
+      </c>
+      <c r="G69" s="8" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H69" s="8" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="I69" s="8" t="inlineStr">
+        <is>
+          <t>Which chapter focuses on reducing branch costs with advanced branch prediction techniques?</t>
+        </is>
+      </c>
+      <c r="J69" s="8" t="inlineStr">
+        <is>
+          <t>Chapter 3.3 focuses on reducing branch costs with advanced branch prediction techniques. This section explores how advanced branch prediction methods can minimize the negative impact of branches on instruction-level parallelism by predicting the most likely branch outcomes, thereby reducing branch mispredictions and associated costs.</t>
+        </is>
+      </c>
+      <c r="K69" s="8" t="inlineStr">
+        <is>
+          <t>source_38.pdf, source_12.pdf</t>
+        </is>
+      </c>
+      <c r="L69" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="M69" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="N69" s="8" t="n">
+        <v>1.67</v>
+      </c>
+      <c r="O69" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="P69" s="8" t="inlineStr"/>
+      <c r="Q69" s="8" t="inlineStr"/>
+      <c r="R69" s="8" t="inlineStr"/>
+      <c r="S69" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-16 14:30</t>
+        </is>
+      </c>
+      <c r="T69" s="8" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+    </row>
+    <row r="70" ht="80" customHeight="1">
+      <c r="A70" s="7" t="inlineStr">
+        <is>
+          <t>E-CO-068</t>
+        </is>
+      </c>
+      <c r="B70" s="7" t="inlineStr">
+        <is>
+          <t>computer_architecture</t>
+        </is>
+      </c>
+      <c r="C70" s="7" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D70" s="7" t="inlineStr">
+        <is>
+          <t>recall</t>
+        </is>
+      </c>
+      <c r="E70" s="7" t="inlineStr">
+        <is>
+          <t>RISC vs CISC architecture</t>
+        </is>
+      </c>
+      <c r="F70" s="7" t="inlineStr">
+        <is>
+          <t>explicit</t>
+        </is>
+      </c>
+      <c r="G70" s="7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H70" s="7" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="I70" s="7" t="inlineStr">
+        <is>
+          <t>What does the text suggest is more important than differentiating between RISC and CISC technologies?</t>
+        </is>
+      </c>
+      <c r="J70" s="7" t="inlineStr">
+        <is>
+          <t>The text suggests that the speed of executing instructions and the performance of running existing software are more important than differentiating between RISC and CISC technologies. Both types of architectures are suitable for their specific applications, but what truly distinguishes them in competition is their ability to execute instructions efficiently and support current software requirements.</t>
+        </is>
+      </c>
+      <c r="K70" s="7" t="inlineStr">
+        <is>
+          <t>source_29.pdf, source_32.pdf, source_30.pdf, source_6.pdf, source_23.pdf, source_24.pdf, source_38.pdf, source_25.pdf, source_27.pdf, source_28.pdf, source_9.pdf, source_26.pdf, source_12.pdf</t>
+        </is>
+      </c>
+      <c r="L70" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="M70" s="7" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="N70" s="7" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="O70" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="P70" s="7" t="inlineStr"/>
+      <c r="Q70" s="7" t="inlineStr"/>
+      <c r="R70" s="7" t="inlineStr"/>
+      <c r="S70" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-16 14:31</t>
+        </is>
+      </c>
+      <c r="T70" s="7" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+    </row>
+    <row r="71" ht="80" customHeight="1">
+      <c r="A71" s="8" t="inlineStr">
+        <is>
+          <t>E-CO-069</t>
+        </is>
+      </c>
+      <c r="B71" s="8" t="inlineStr">
+        <is>
+          <t>computer_architecture</t>
+        </is>
+      </c>
+      <c r="C71" s="8" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D71" s="8" t="inlineStr">
+        <is>
+          <t>recall</t>
+        </is>
+      </c>
+      <c r="E71" s="8" t="inlineStr">
+        <is>
+          <t>Virtual memory and address translation</t>
+        </is>
+      </c>
+      <c r="F71" s="8" t="inlineStr">
+        <is>
+          <t>explicit</t>
+        </is>
+      </c>
+      <c r="G71" s="8" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H71" s="8" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="I71" s="8" t="inlineStr">
+        <is>
+          <t>What does the term "address translation" refer to in the context of virtual memory, and how does it involve both hardware and software?</t>
+        </is>
+      </c>
+      <c r="J71" s="8" t="inlineStr">
+        <is>
+          <t>Address translation in the context of virtual memory refers to the process where the processor generates virtual addresses that are then converted into physical addresses through a combination of hardware and software mechanisms. This translation ensures that the processor can access the correct location in main memory based on the virtual addresses assigned by the operating system, thus facilitating the management of a very large address space.</t>
+        </is>
+      </c>
+      <c r="K71" s="8" t="inlineStr">
+        <is>
+          <t>source_32.pdf, source_30.pdf, source_23.pdf, source_38.pdf, source_27.pdf, source_25.pdf, source_28.pdf, source_9.pdf, source_26.pdf, source_12.pdf</t>
+        </is>
+      </c>
+      <c r="L71" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="M71" s="8" t="n">
+        <v>4.25</v>
+      </c>
+      <c r="N71" s="8" t="n">
+        <v>3</v>
+      </c>
+      <c r="O71" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="P71" s="8" t="inlineStr"/>
+      <c r="Q71" s="8" t="inlineStr"/>
+      <c r="R71" s="8" t="inlineStr"/>
+      <c r="S71" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-16 14:31</t>
+        </is>
+      </c>
+      <c r="T71" s="8" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+    </row>
+    <row r="72" ht="80" customHeight="1">
+      <c r="A72" s="7" t="inlineStr">
+        <is>
+          <t>E-CO-070</t>
+        </is>
+      </c>
+      <c r="B72" s="7" t="inlineStr">
+        <is>
+          <t>computer_architecture</t>
+        </is>
+      </c>
+      <c r="C72" s="7" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D72" s="7" t="inlineStr">
+        <is>
+          <t>recall</t>
+        </is>
+      </c>
+      <c r="E72" s="7" t="inlineStr">
+        <is>
+          <t>Multicore processors and parallelism</t>
+        </is>
+      </c>
+      <c r="F72" s="7" t="inlineStr">
+        <is>
+          <t>explicit</t>
+        </is>
+      </c>
+      <c r="G72" s="7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H72" s="7" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="I72" s="7" t="inlineStr">
+        <is>
+          <t>In a single-issue in-order pipeline where all instructions take three cycles to complete (Fetch, Decode, Register file read), how many cycles would it take to fully execute a sequence of 10 integer operations in parallel on a multicore processor exploiting thread-level parallelism?</t>
+        </is>
+      </c>
+      <c r="J72" s="7" t="inlineStr">
+        <is>
+          <t>Given the single-issue in-order pipeline where each instruction takes three cycles to complete, and assuming the multicore processor can fully exploit thread-level parallelism to run ten integer operations in parallel, it would take a total of 3 cycles to fully execute the sequence of 10 integer operations. This is because the parallel execution of these operations simultaneously reduces the time required to their minimum cycle count, which is determined by the longest pipeline stage, in this case, three cycles.</t>
+        </is>
+      </c>
+      <c r="K72" s="7" t="inlineStr">
+        <is>
+          <t>source_38.pdf, source_6.pdf, source_12.pdf</t>
+        </is>
+      </c>
+      <c r="L72" s="7" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="M72" s="7" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="N72" s="7" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="O72" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="P72" s="7" t="inlineStr"/>
+      <c r="Q72" s="7" t="inlineStr"/>
+      <c r="R72" s="7" t="inlineStr"/>
+      <c r="S72" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-16 14:32</t>
+        </is>
+      </c>
+      <c r="T72" s="7" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+    </row>
+    <row r="73" ht="80" customHeight="1">
+      <c r="A73" s="8" t="inlineStr">
+        <is>
+          <t>E-CO-071</t>
+        </is>
+      </c>
+      <c r="B73" s="8" t="inlineStr">
+        <is>
+          <t>computer_architecture</t>
+        </is>
+      </c>
+      <c r="C73" s="8" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D73" s="8" t="inlineStr">
+        <is>
+          <t>recall</t>
+        </is>
+      </c>
+      <c r="E73" s="8" t="inlineStr">
+        <is>
+          <t>Amdahl's law and performance limits</t>
+        </is>
+      </c>
+      <c r="F73" s="8" t="inlineStr">
+        <is>
+          <t>explicit</t>
+        </is>
+      </c>
+      <c r="G73" s="8" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H73" s="8" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="I73" s="8" t="inlineStr">
+        <is>
+          <t>What is the theoretical maximum speedup you can achieve if 90% of the application is parallelizable, according to Amdahl's Law?</t>
+        </is>
+      </c>
+      <c r="J73" s="8" t="inlineStr">
+        <is>
+          <t>According to Amdahl's Law, the theoretical maximum speedup achievable when 90% of the application is parallelizable is theoretically unlimited, as the formula \( \text{Speedup} = \frac{1}{(1 - p) + \frac{p}{N}} \) approaches infinity as \( p \) (the parallelizable fraction) increases towards 1, where \( p = 0.90 \) and \( N \) represents the number of processors. However, in practical scenarios, the speedup is constrained by the remaining 10% of the application that cannot be parallelized.</t>
+        </is>
+      </c>
+      <c r="K73" s="8" t="inlineStr">
+        <is>
+          <t>source_28.pdf, source_38.pdf, source_30.pdf, source_12.pdf</t>
+        </is>
+      </c>
+      <c r="L73" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="M73" s="8" t="n">
+        <v>4.25</v>
+      </c>
+      <c r="N73" s="8" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="O73" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="P73" s="8" t="inlineStr"/>
+      <c r="Q73" s="8" t="inlineStr"/>
+      <c r="R73" s="8" t="inlineStr"/>
+      <c r="S73" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-16 14:32</t>
+        </is>
+      </c>
+      <c r="T73" s="8" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+    </row>
+    <row r="74" ht="80" customHeight="1">
+      <c r="A74" s="7" t="inlineStr">
+        <is>
+          <t>E-CO-072</t>
+        </is>
+      </c>
+      <c r="B74" s="7" t="inlineStr">
+        <is>
+          <t>computer_architecture</t>
+        </is>
+      </c>
+      <c r="C74" s="7" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D74" s="7" t="inlineStr">
+        <is>
+          <t>recall</t>
+        </is>
+      </c>
+      <c r="E74" s="7" t="inlineStr">
+        <is>
+          <t>Direct memory access</t>
+        </is>
+      </c>
+      <c r="F74" s="7" t="inlineStr">
+        <is>
+          <t>explicit</t>
+        </is>
+      </c>
+      <c r="G74" s="7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H74" s="7" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="I74" s="7" t="inlineStr">
+        <is>
+          <t>Which paper discusses the use of a memory conflict buffer for dynamic memory disambiguation?</t>
+        </is>
+      </c>
+      <c r="J74" s="7" t="inlineStr">
+        <is>
+          <t>The paper that discusses the use of a memory conflict buffer for dynamic memory disambiguation is "Dynamic memory disambiguation using the memory conflict buffer" by Gallagher et al., presented at the Sixth International Conference on Architectural Support for Programming Languages and Operating Systems (ASPLOS) in 1994.</t>
+        </is>
+      </c>
+      <c r="K74" s="7" t="inlineStr">
+        <is>
+          <t>source_38.pdf, source_9.pdf, source_12.pdf</t>
+        </is>
+      </c>
+      <c r="L74" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="M74" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="N74" s="7" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="O74" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="P74" s="7" t="inlineStr"/>
+      <c r="Q74" s="7" t="inlineStr"/>
+      <c r="R74" s="7" t="inlineStr"/>
+      <c r="S74" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-16 14:33</t>
+        </is>
+      </c>
+      <c r="T74" s="7" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+    </row>
+    <row r="75" ht="80" customHeight="1">
+      <c r="A75" s="8" t="inlineStr">
+        <is>
+          <t>E-CO-073</t>
+        </is>
+      </c>
+      <c r="B75" s="8" t="inlineStr">
+        <is>
+          <t>computer_architecture</t>
+        </is>
+      </c>
+      <c r="C75" s="8" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D75" s="8" t="inlineStr">
+        <is>
+          <t>recall</t>
+        </is>
+      </c>
+      <c r="E75" s="8" t="inlineStr">
+        <is>
+          <t>Bus architecture and interconnects</t>
+        </is>
+      </c>
+      <c r="F75" s="8" t="inlineStr">
+        <is>
+          <t>explicit</t>
+        </is>
+      </c>
+      <c r="G75" s="8" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H75" s="8" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="I75" s="8" t="inlineStr">
+        <is>
+          <t>What term describes the process where a device identifies the location of requested information using an address?</t>
+        </is>
+      </c>
+      <c r="J75" s="8" t="inlineStr">
+        <is>
+          <t>The term that describes the process where a device identifies the location of requested information using an address is simply referred to as addressing. This mechanism allows the receiver to pinpoint the exact location of the sought-after data within the interconnection network.</t>
+        </is>
+      </c>
+      <c r="K75" s="8" t="inlineStr">
+        <is>
+          <t>source_44.pdf, source_29.pdf, source_32.pdf, source_30.pdf, source_23.pdf, source_24.pdf, source_38.pdf, source_27.pdf, source_25.pdf, source_28.pdf, source_9.pdf, source_26.pdf, source_12.pdf</t>
+        </is>
+      </c>
+      <c r="L75" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="M75" s="8" t="n">
+        <v>4.25</v>
+      </c>
+      <c r="N75" s="8" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="O75" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="P75" s="8" t="inlineStr"/>
+      <c r="Q75" s="8" t="inlineStr"/>
+      <c r="R75" s="8" t="inlineStr"/>
+      <c r="S75" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-16 14:33</t>
+        </is>
+      </c>
+      <c r="T75" s="8" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" ht="80" customHeight="1">
+      <c r="A76" s="7" t="inlineStr">
+        <is>
+          <t>E-CO-074</t>
+        </is>
+      </c>
+      <c r="B76" s="7" t="inlineStr">
+        <is>
+          <t>computer_architecture</t>
+        </is>
+      </c>
+      <c r="C76" s="7" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D76" s="7" t="inlineStr">
+        <is>
+          <t>recall</t>
+        </is>
+      </c>
+      <c r="E76" s="7" t="inlineStr">
+        <is>
+          <t>Floating point representation</t>
+        </is>
+      </c>
+      <c r="F76" s="7" t="inlineStr">
+        <is>
+          <t>explicit</t>
+        </is>
+      </c>
+      <c r="G76" s="7" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H76" s="7" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="I76" s="7" t="inlineStr">
+        <is>
+          <t>What is the largest number that can be represented in IEEE single-precision floating-point format, and how would you represent it in binary form?</t>
+        </is>
+      </c>
+      <c r="J76" s="7" t="inlineStr">
+        <is>
+          <t>The largest number that can be represented in IEEE single-precision floating-point format is approximately 3.4028235 × 10^38. In binary form, this number is represented as 0x7F7FFFFF, which corresponds to the maximum exponent and all 23 mantissa bits set to 1.</t>
+        </is>
+      </c>
+      <c r="K76" s="7" t="inlineStr">
+        <is>
+          <t>source_27.pdf, source_12.pdf</t>
+        </is>
+      </c>
+      <c r="L76" s="7" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="M76" s="7" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="N76" s="7" t="n">
+        <v>2.33</v>
+      </c>
+      <c r="O76" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="P76" s="7" t="inlineStr"/>
+      <c r="Q76" s="7" t="inlineStr"/>
+      <c r="R76" s="7" t="inlineStr"/>
+      <c r="S76" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-16 14:34</t>
+        </is>
+      </c>
+      <c r="T76" s="7" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" ht="80" customHeight="1">
+      <c r="A77" s="8" t="inlineStr">
+        <is>
+          <t>E-CO-075</t>
+        </is>
+      </c>
+      <c r="B77" s="8" t="inlineStr">
+        <is>
+          <t>computer_architecture</t>
+        </is>
+      </c>
+      <c r="C77" s="8" t="inlineStr">
+        <is>
+          <t>easy</t>
+        </is>
+      </c>
+      <c r="D77" s="8" t="inlineStr">
+        <is>
+          <t>recall</t>
+        </is>
+      </c>
+      <c r="E77" s="8" t="inlineStr">
+        <is>
+          <t>Assembly language and low level programming</t>
+        </is>
+      </c>
+      <c r="F77" s="8" t="inlineStr">
+        <is>
+          <t>explicit</t>
+        </is>
+      </c>
+      <c r="G77" s="8" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="H77" s="8" t="inlineStr">
+        <is>
+          <t>0.8</t>
+        </is>
+      </c>
+      <c r="I77" s="8" t="inlineStr">
+        <is>
+          <t>Which of the following instruction set architectures (ISA) is characterized by narrow instructions that support fewer operations, smaller address and immediate fields, fewer registers, and a two-address format, and what does the "C" in RV32IC stand for?</t>
+        </is>
+      </c>
+      <c r="J77" s="8" t="inlineStr">
+        <is>
+          <t>The instruction set architecture characterized by narrow instructions that support fewer operations, smaller address and immediate fields, fewer registers, and a two-address format is RISC (Reduced Instruction Set Computing). The "C" in RV32IC stands for "compressed," indicating that common instruction occurrences are encoded in 16-bit formats to optimize space and efficiency.</t>
+        </is>
+      </c>
+      <c r="K77" s="8" t="inlineStr">
+        <is>
+          <t>source_30.pdf, source_23.pdf, source_24.pdf, source_38.pdf, source_9.pdf, source_12.pdf</t>
+        </is>
+      </c>
+      <c r="L77" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="M77" s="8" t="n">
+        <v>4.25</v>
+      </c>
+      <c r="N77" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="O77" s="8" t="n">
+        <v>1</v>
+      </c>
+      <c r="P77" s="8" t="inlineStr"/>
+      <c r="Q77" s="8" t="inlineStr"/>
+      <c r="R77" s="8" t="inlineStr"/>
+      <c r="S77" s="8" t="inlineStr">
+        <is>
+          <t>2026-05-16 14:35</t>
+        </is>
+      </c>
+      <c r="T77" s="8" t="inlineStr">
+        <is>
+          <t>done</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="7">
     <mergeCell ref="A1:D1"/>

</xml_diff>